<commit_message>
added maybe unused command
</commit_message>
<xml_diff>
--- a/docs/roadmap/Roadmap - C++ New Features.xlsx
+++ b/docs/roadmap/Roadmap - C++ New Features.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Hadi\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\git\Cpp-Modern-Features\docs\roadmap\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C91E6525-7D4C-43FD-9040-CF5FC88D76C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8B401A7-7921-49DA-A71C-B5A07446CB84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="C++11" sheetId="3" r:id="rId1"/>
@@ -31,15 +31,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="384" uniqueCount="343">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="382" uniqueCount="342">
   <si>
     <t>[[deprecated]]</t>
   </si>
   <si>
     <t>Hadi Abbasi</t>
-  </si>
-  <si>
-    <t>std::make_shared</t>
   </si>
   <si>
     <t xml:space="preserve"> enum class</t>
@@ -1394,7 +1391,7 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
@@ -1402,7 +1399,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B2" t="s">
         <v>1</v>
@@ -1410,7 +1407,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B3" t="s">
         <v>1</v>
@@ -1418,7 +1415,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B4" t="s">
         <v>1</v>
@@ -1426,7 +1423,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B5" t="s">
         <v>1</v>
@@ -1434,7 +1431,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B6" t="s">
         <v>1</v>
@@ -1442,7 +1439,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B7" t="s">
         <v>1</v>
@@ -1450,7 +1447,7 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B8" t="s">
         <v>1</v>
@@ -1458,60 +1455,60 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B18" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
   </sheetData>
@@ -1521,7 +1518,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2022B5AF-BBCF-4D30-980F-26F615A31FDF}">
-  <dimension ref="A1:Z20"/>
+  <dimension ref="A1:Z19"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="45.21875" customWidth="1"/>
@@ -1539,10 +1536,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2" t="s">
-        <v>1</v>
+        <v>22</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
@@ -1628,11 +1622,6 @@
     <row r="19" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>39</v>
-      </c>
-    </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A20" t="s">
-        <v>40</v>
       </c>
     </row>
   </sheetData>
@@ -1652,247 +1641,247 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B2" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B5" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B6" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B7" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B8" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B9" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
+        <v>49</v>
+      </c>
+      <c r="B10" t="s">
         <v>50</v>
-      </c>
-      <c r="B10" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
   </sheetData>
@@ -1912,322 +1901,322 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="54" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="55" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="56" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="57" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="58" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="59" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="60" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="61" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="62" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="63" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="64" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
   </sheetData>
@@ -2247,252 +2236,252 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
   </sheetData>
@@ -2512,837 +2501,837 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="54" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
     </row>
     <row r="55" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
     </row>
     <row r="56" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
     </row>
     <row r="57" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="58" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="59" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="60" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
     </row>
     <row r="61" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="62" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
     </row>
     <row r="63" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="64" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
     </row>
     <row r="65" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
     </row>
     <row r="66" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="67" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
     </row>
     <row r="68" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
     </row>
     <row r="69" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="70" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
     </row>
     <row r="71" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
     </row>
     <row r="72" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
     </row>
     <row r="73" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
     </row>
     <row r="74" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="75" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
     </row>
     <row r="76" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
     </row>
     <row r="77" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
     </row>
     <row r="78" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="79" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="80" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="81" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="82" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="83" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="84" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="85" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
     </row>
     <row r="86" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
     </row>
     <row r="87" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
     </row>
     <row r="88" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
     </row>
     <row r="89" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
     </row>
     <row r="90" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="91" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="92" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="93" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="94" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
     </row>
     <row r="95" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
     </row>
     <row r="96" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
     </row>
     <row r="97" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
     </row>
     <row r="98" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
     </row>
     <row r="99" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
     </row>
     <row r="100" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
     </row>
     <row r="101" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
     </row>
     <row r="102" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
     </row>
     <row r="103" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
     </row>
     <row r="104" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
     </row>
     <row r="105" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
     </row>
     <row r="106" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
     </row>
     <row r="107" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
     </row>
     <row r="108" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
     </row>
     <row r="109" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A109" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
     </row>
     <row r="110" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
     </row>
     <row r="111" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
     </row>
     <row r="112" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="113" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="114" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A114" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
     </row>
     <row r="115" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A115" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
     </row>
     <row r="116" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A116" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
     </row>
     <row r="117" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A117" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
     </row>
     <row r="118" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A118" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
     </row>
     <row r="119" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A119" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
     </row>
     <row r="120" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A120" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
     </row>
     <row r="121" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A121" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="122" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A122" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="123" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A123" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
     </row>
     <row r="124" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A124" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
     </row>
     <row r="125" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A125" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
     </row>
     <row r="126" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A126" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
     </row>
     <row r="127" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A127" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
     </row>
     <row r="128" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A128" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
     </row>
     <row r="129" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A129" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
     </row>
     <row r="130" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A130" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
     </row>
     <row r="131" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A131" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
     </row>
     <row r="132" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A132" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
     </row>
     <row r="133" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A133" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
     </row>
     <row r="134" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A134" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
     </row>
     <row r="135" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A135" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
     </row>
     <row r="136" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A136" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
     </row>
     <row r="137" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A137" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
     </row>
     <row r="138" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A138" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
     </row>
     <row r="139" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A139" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
     </row>
     <row r="140" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A140" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="141" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A141" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
     </row>
     <row r="142" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A142" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="143" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A143" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
     </row>
     <row r="144" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A144" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
     </row>
     <row r="145" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A145" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
     </row>
     <row r="146" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A146" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
     </row>
     <row r="147" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A147" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
     </row>
     <row r="148" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A148" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
     </row>
     <row r="149" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A149" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
     </row>
     <row r="150" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A150" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
     </row>
     <row r="151" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A151" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
     </row>
     <row r="152" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A152" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
     </row>
     <row r="153" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A153" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
     </row>
     <row r="154" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A154" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
     </row>
     <row r="155" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A155" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
     </row>
     <row r="156" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A156" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="157" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A157" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
     </row>
     <row r="158" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A158" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
     </row>
     <row r="159" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A159" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
     </row>
     <row r="160" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A160" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
     </row>
     <row r="161" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A161" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
     </row>
     <row r="162" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A162" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
     </row>
     <row r="163" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A163" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
     </row>
     <row r="164" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A164" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
     </row>
     <row r="165" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A165" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
     </row>
     <row r="166" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A166" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
     </row>
     <row r="167" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A167" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs added for generic lambda and lambda init-capture
</commit_message>
<xml_diff>
--- a/docs/roadmap/Roadmap - C++ New Features.xlsx
+++ b/docs/roadmap/Roadmap - C++ New Features.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\git\Cpp-Modern-Features\docs\roadmap\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8B401A7-7921-49DA-A71C-B5A07446CB84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A62EAB4-8540-493C-B6D0-4156400EAC4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,10 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="382" uniqueCount="342">
-  <si>
-    <t>[[deprecated]]</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="382" uniqueCount="340">
   <si>
     <t>Hadi Abbasi</t>
   </si>
@@ -97,9 +94,6 @@
   </si>
   <si>
     <t>Mohammad</t>
-  </si>
-  <si>
-    <t>generic lambda</t>
   </si>
   <si>
     <t>lambda init-capture</t>
@@ -1391,124 +1385,124 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B1" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B2" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B3" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B4" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B5" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B6" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B7" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B8" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B18" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
   </sheetData>
@@ -1518,7 +1512,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2022B5AF-BBCF-4D30-980F-26F615A31FDF}">
-  <dimension ref="A1:Z19"/>
+  <dimension ref="A1:Z17"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="45.21875" customWidth="1"/>
@@ -1528,10 +1522,10 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B1" t="s">
         <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
@@ -1578,6 +1572,9 @@
       <c r="A10" t="s">
         <v>30</v>
       </c>
+      <c r="B10" t="s">
+        <v>0</v>
+      </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
@@ -1598,6 +1595,9 @@
       <c r="A14" t="s">
         <v>34</v>
       </c>
+      <c r="B14" t="s">
+        <v>0</v>
+      </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
@@ -1612,16 +1612,6 @@
     <row r="17" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>37</v>
-      </c>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A18" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A19" t="s">
-        <v>39</v>
       </c>
     </row>
   </sheetData>
@@ -1641,247 +1631,247 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B2" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B3" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B4" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B5" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B6" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B7" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B8" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
+        <v>46</v>
+      </c>
+      <c r="B9" t="s">
         <v>48</v>
-      </c>
-      <c r="B9" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B10" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
   </sheetData>
@@ -1901,322 +1891,322 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
     </row>
     <row r="54" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
     </row>
     <row r="55" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="56" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="57" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
     </row>
     <row r="58" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="59" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
     </row>
     <row r="60" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
     </row>
     <row r="61" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
     </row>
     <row r="62" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
     </row>
     <row r="63" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
     </row>
     <row r="64" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
     </row>
   </sheetData>
@@ -2236,252 +2226,252 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
     </row>
   </sheetData>
@@ -2501,837 +2491,837 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
     </row>
     <row r="54" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
     </row>
     <row r="55" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
     </row>
     <row r="56" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
     </row>
     <row r="57" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
     </row>
     <row r="58" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
     </row>
     <row r="59" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
     </row>
     <row r="60" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
     </row>
     <row r="61" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
     </row>
     <row r="62" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
     </row>
     <row r="63" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
     </row>
     <row r="64" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
     </row>
     <row r="65" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
     </row>
     <row r="66" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="67" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
     </row>
     <row r="68" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
     </row>
     <row r="69" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
     </row>
     <row r="70" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
     </row>
     <row r="71" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
     </row>
     <row r="72" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="73" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
     </row>
     <row r="74" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="75" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
     </row>
     <row r="76" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
     </row>
     <row r="77" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
     </row>
     <row r="78" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
     </row>
     <row r="79" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
     </row>
     <row r="80" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
     </row>
     <row r="81" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
     </row>
     <row r="82" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
     </row>
     <row r="83" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
     </row>
     <row r="84" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="85" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
     </row>
     <row r="86" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
     </row>
     <row r="87" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
     </row>
     <row r="88" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
     </row>
     <row r="89" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
     </row>
     <row r="90" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
     </row>
     <row r="91" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
     </row>
     <row r="92" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
     </row>
     <row r="93" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
     </row>
     <row r="94" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
     </row>
     <row r="95" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
     </row>
     <row r="96" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
     </row>
     <row r="97" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="98" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
     </row>
     <row r="99" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
     </row>
     <row r="100" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
     </row>
     <row r="101" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
     </row>
     <row r="102" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
     </row>
     <row r="103" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
     </row>
     <row r="104" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
     </row>
     <row r="105" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
     </row>
     <row r="106" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
     </row>
     <row r="107" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
     </row>
     <row r="108" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
     </row>
     <row r="109" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A109" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
     </row>
     <row r="110" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
     </row>
     <row r="111" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
     </row>
     <row r="112" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
     </row>
     <row r="113" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
     </row>
     <row r="114" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A114" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
     </row>
     <row r="115" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A115" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
     </row>
     <row r="116" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A116" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
     </row>
     <row r="117" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A117" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
     </row>
     <row r="118" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A118" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
     </row>
     <row r="119" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A119" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
     </row>
     <row r="120" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A120" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
     </row>
     <row r="121" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A121" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
     </row>
     <row r="122" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A122" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
     </row>
     <row r="123" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A123" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
     </row>
     <row r="124" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A124" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
     </row>
     <row r="125" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A125" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
     </row>
     <row r="126" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A126" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
     </row>
     <row r="127" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A127" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
     </row>
     <row r="128" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A128" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
     </row>
     <row r="129" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A129" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
     </row>
     <row r="130" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A130" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
     </row>
     <row r="131" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A131" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
     </row>
     <row r="132" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A132" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
     </row>
     <row r="133" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A133" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
     </row>
     <row r="134" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A134" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
     </row>
     <row r="135" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A135" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
     </row>
     <row r="136" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A136" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
     </row>
     <row r="137" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A137" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
     </row>
     <row r="138" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A138" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
     </row>
     <row r="139" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A139" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
     </row>
     <row r="140" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A140" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
     </row>
     <row r="141" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A141" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
     </row>
     <row r="142" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A142" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
     </row>
     <row r="143" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A143" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
     </row>
     <row r="144" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A144" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
     </row>
     <row r="145" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A145" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
     </row>
     <row r="146" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A146" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
     </row>
     <row r="147" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A147" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
     </row>
     <row r="148" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A148" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
     </row>
     <row r="149" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A149" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
     </row>
     <row r="150" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A150" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
     </row>
     <row r="151" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A151" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
     </row>
     <row r="152" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A152" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
     </row>
     <row r="153" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A153" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
     </row>
     <row r="154" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A154" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
     </row>
     <row r="155" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A155" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
     </row>
     <row r="156" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A156" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
     </row>
     <row r="157" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A157" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
     </row>
     <row r="158" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A158" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
     </row>
     <row r="159" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A159" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
     </row>
     <row r="160" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A160" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
     </row>
     <row r="161" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A161" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
     </row>
     <row r="162" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A162" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
     </row>
     <row r="163" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A163" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
     </row>
     <row r="164" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A164" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
     </row>
     <row r="165" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A165" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
     </row>
     <row r="166" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A166" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
     </row>
     <row r="167" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A167" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added the tutorial of putting details tag in md file inside roadmap directory
</commit_message>
<xml_diff>
--- a/docs/roadmap/Roadmap - C++ New Features.xlsx
+++ b/docs/roadmap/Roadmap - C++ New Features.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\git\Cpp-Modern-Features\docs\roadmap\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A62EAB4-8540-493C-B6D0-4156400EAC4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F98E6030-C8B8-4ACD-8884-6017350EADCE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="C++11" sheetId="3" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="382" uniqueCount="340">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="380" uniqueCount="339">
   <si>
     <t>Hadi Abbasi</t>
   </si>
@@ -94,9 +94,6 @@
   </si>
   <si>
     <t>Mohammad</t>
-  </si>
-  <si>
-    <t>lambda init-capture</t>
   </si>
   <si>
     <t>return type deduction</t>
@@ -1512,7 +1509,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2022B5AF-BBCF-4D30-980F-26F615A31FDF}">
-  <dimension ref="A1:Z17"/>
+  <dimension ref="A1:Z16"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="45.21875" customWidth="1"/>
@@ -1524,9 +1521,6 @@
       <c r="A1" t="s">
         <v>21</v>
       </c>
-      <c r="B1" t="s">
-        <v>0</v>
-      </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
@@ -1567,14 +1561,14 @@
       <c r="A9" t="s">
         <v>29</v>
       </c>
+      <c r="B9" t="s">
+        <v>0</v>
+      </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>30</v>
       </c>
-      <c r="B10" t="s">
-        <v>0</v>
-      </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
@@ -1590,14 +1584,14 @@
       <c r="A13" t="s">
         <v>33</v>
       </c>
+      <c r="B13" t="s">
+        <v>0</v>
+      </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>34</v>
       </c>
-      <c r="B14" t="s">
-        <v>0</v>
-      </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
@@ -1607,11 +1601,6 @@
     <row r="16" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>36</v>
-      </c>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A17" t="s">
-        <v>37</v>
       </c>
     </row>
   </sheetData>
@@ -1631,247 +1620,247 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B5" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B6" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B7" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B8" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B9" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
+        <v>46</v>
+      </c>
+      <c r="B10" t="s">
         <v>47</v>
-      </c>
-      <c r="B10" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
   </sheetData>
@@ -1891,322 +1880,322 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="54" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="55" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="56" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="57" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="58" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="59" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="60" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="61" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="62" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="63" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="64" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
   </sheetData>
@@ -2226,252 +2215,252 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
   </sheetData>
@@ -2491,837 +2480,837 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
     </row>
     <row r="54" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
     </row>
     <row r="55" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
     </row>
     <row r="56" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="57" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
     </row>
     <row r="58" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
     </row>
     <row r="59" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
     </row>
     <row r="60" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="61" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="62" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="63" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
     </row>
     <row r="64" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="65" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
     </row>
     <row r="66" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="67" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
     </row>
     <row r="68" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
     </row>
     <row r="69" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="70" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
     </row>
     <row r="71" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
     </row>
     <row r="72" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="73" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
     </row>
     <row r="74" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
     </row>
     <row r="75" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
     </row>
     <row r="76" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
     </row>
     <row r="77" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="78" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
     </row>
     <row r="79" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
     </row>
     <row r="80" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
     </row>
     <row r="81" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="82" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="83" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="84" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="85" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="86" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="87" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="88" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
     </row>
     <row r="89" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
     </row>
     <row r="90" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
     </row>
     <row r="91" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
     </row>
     <row r="92" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
     </row>
     <row r="93" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="94" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="95" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="96" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="97" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="98" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
     </row>
     <row r="99" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
     </row>
     <row r="100" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
     </row>
     <row r="101" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
     </row>
     <row r="102" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
     </row>
     <row r="103" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
     </row>
     <row r="104" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
     </row>
     <row r="105" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
     </row>
     <row r="106" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
     </row>
     <row r="107" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
     </row>
     <row r="108" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
     </row>
     <row r="109" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A109" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
     </row>
     <row r="110" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
     </row>
     <row r="111" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
     </row>
     <row r="112" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
     </row>
     <row r="113" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
     </row>
     <row r="114" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A114" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
     </row>
     <row r="115" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A115" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="116" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A116" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="117" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A117" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
     </row>
     <row r="118" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A118" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
     </row>
     <row r="119" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A119" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
     </row>
     <row r="120" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A120" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
     </row>
     <row r="121" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A121" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="122" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A122" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
     </row>
     <row r="123" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A123" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
     </row>
     <row r="124" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A124" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
     </row>
     <row r="125" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A125" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
     </row>
     <row r="126" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A126" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
     </row>
     <row r="127" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A127" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
     </row>
     <row r="128" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A128" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
     </row>
     <row r="129" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A129" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
     </row>
     <row r="130" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A130" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
     </row>
     <row r="131" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A131" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
     </row>
     <row r="132" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A132" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
     </row>
     <row r="133" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A133" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
     </row>
     <row r="134" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A134" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
     </row>
     <row r="135" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A135" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
     </row>
     <row r="136" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A136" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
     </row>
     <row r="137" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A137" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
     </row>
     <row r="138" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A138" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
     </row>
     <row r="139" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A139" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
     </row>
     <row r="140" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A140" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
     </row>
     <row r="141" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A141" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
     </row>
     <row r="142" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A142" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
     </row>
     <row r="143" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A143" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
     </row>
     <row r="144" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A144" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
     </row>
     <row r="145" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A145" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
     </row>
     <row r="146" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A146" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="147" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A147" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
     </row>
     <row r="148" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A148" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="149" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A149" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
     </row>
     <row r="150" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A150" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
     </row>
     <row r="151" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A151" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
     </row>
     <row r="152" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A152" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
     </row>
     <row r="153" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A153" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
     </row>
     <row r="154" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A154" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
     </row>
     <row r="155" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A155" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
     </row>
     <row r="156" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A156" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
     </row>
     <row r="157" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A157" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
     </row>
     <row r="158" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A158" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
     </row>
     <row r="159" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A159" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
     </row>
     <row r="160" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A160" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
     </row>
     <row r="161" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A161" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
     </row>
     <row r="162" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A162" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="163" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A163" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
     </row>
     <row r="164" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A164" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
     </row>
     <row r="165" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A165" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
     </row>
     <row r="166" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A166" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
     </row>
     <row r="167" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A167" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added default-delete,enum class, final , noexcept
</commit_message>
<xml_diff>
--- a/docs/roadmap/Roadmap - C++ New Features.xlsx
+++ b/docs/roadmap/Roadmap - C++ New Features.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\git\Cpp-Modern-Features\docs\roadmap\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F98E6030-C8B8-4ACD-8884-6017350EADCE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CFD8D7F4-6C49-42F3-8BD4-D95C2682F245}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,23 +31,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="380" uniqueCount="339">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="374" uniqueCount="334">
   <si>
     <t>Hadi Abbasi</t>
   </si>
   <si>
-    <t xml:space="preserve"> enum class</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> noexcept</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> final</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> default / delete</t>
-  </si>
-  <si>
     <t>variadic templates</t>
   </si>
   <si>
@@ -66,15 +54,6 @@
     <t xml:space="preserve"> std::begin / std::end</t>
   </si>
   <si>
-    <t xml:space="preserve"> in thread</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> std::lock_guard</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> std::unique_lock</t>
-  </si>
-  <si>
     <t xml:space="preserve"> std::random</t>
   </si>
   <si>
@@ -1048,6 +1027,12 @@
   </si>
   <si>
     <t>[3]: https://en.cppreference.com/cpp/identifier_with_special_meaning/pre?utm_source=chatgpt.com "C++ identifier with special meaning: pre (since C++26) - cppreference.com"</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> std::lock_guard ( in thread)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> std::unique_lock ( in thread)</t>
   </si>
 </sst>
 </file>
@@ -1372,7 +1357,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0CBDD6F8-296C-4055-8D41-426BC8FCE08A}">
-  <dimension ref="A1:X19"/>
+  <dimension ref="A1:X14"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="28.109375" customWidth="1"/>
@@ -1414,7 +1399,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B5" t="s">
         <v>0</v>
@@ -1422,7 +1407,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>6</v>
+        <v>332</v>
       </c>
       <c r="B6" t="s">
         <v>0</v>
@@ -1430,7 +1415,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>7</v>
+        <v>333</v>
       </c>
       <c r="B7" t="s">
         <v>0</v>
@@ -1438,68 +1423,40 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>8</v>
-      </c>
-      <c r="B8" t="s">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
+        <v>11</v>
+      </c>
+      <c r="B13" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A16" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A17" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A18" t="s">
-        <v>18</v>
-      </c>
-      <c r="B18" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A19" t="s">
-        <v>19</v>
+        <v>12</v>
       </c>
     </row>
   </sheetData>
@@ -1519,47 +1476,47 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>21</v>
+        <v>14</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>23</v>
+        <v>16</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>26</v>
+        <v>19</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="B9" t="s">
         <v>0</v>
@@ -1567,22 +1524,22 @@
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>31</v>
+        <v>24</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>32</v>
+        <v>25</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="B13" t="s">
         <v>0</v>
@@ -1590,17 +1547,17 @@
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
     </row>
   </sheetData>
@@ -1620,247 +1577,247 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>37</v>
+        <v>30</v>
       </c>
       <c r="B1" t="s">
-        <v>47</v>
+        <v>40</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="B2" t="s">
-        <v>47</v>
+        <v>40</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="B3" t="s">
-        <v>47</v>
+        <v>40</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
+        <v>33</v>
+      </c>
+      <c r="B4" t="s">
         <v>40</v>
-      </c>
-      <c r="B4" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="B5" t="s">
-        <v>47</v>
+        <v>40</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="B6" t="s">
-        <v>47</v>
+        <v>40</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="B7" t="s">
-        <v>47</v>
+        <v>40</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>44</v>
+        <v>37</v>
       </c>
       <c r="B8" t="s">
-        <v>47</v>
+        <v>40</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="B9" t="s">
-        <v>47</v>
+        <v>40</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>46</v>
+        <v>39</v>
       </c>
       <c r="B10" t="s">
-        <v>47</v>
+        <v>40</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>80</v>
+        <v>73</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>79</v>
+        <v>72</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>78</v>
+        <v>71</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>77</v>
+        <v>70</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>76</v>
+        <v>69</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>75</v>
+        <v>68</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>48</v>
+        <v>41</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>49</v>
+        <v>42</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>50</v>
+        <v>43</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>51</v>
+        <v>44</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>52</v>
+        <v>45</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>56</v>
+        <v>49</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>57</v>
+        <v>50</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>58</v>
+        <v>51</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>59</v>
+        <v>52</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>63</v>
+        <v>56</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>66</v>
+        <v>59</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>68</v>
+        <v>61</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>71</v>
+        <v>64</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>73</v>
+        <v>66</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>74</v>
+        <v>67</v>
       </c>
     </row>
   </sheetData>
@@ -1880,322 +1837,322 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>81</v>
+        <v>74</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>82</v>
+        <v>75</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>83</v>
+        <v>76</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>84</v>
+        <v>77</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>85</v>
+        <v>78</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>86</v>
+        <v>79</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>87</v>
+        <v>80</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>88</v>
+        <v>81</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>89</v>
+        <v>82</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>90</v>
+        <v>83</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>91</v>
+        <v>84</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>92</v>
+        <v>85</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>93</v>
+        <v>86</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>94</v>
+        <v>87</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>95</v>
+        <v>88</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>96</v>
+        <v>89</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>97</v>
+        <v>90</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>98</v>
+        <v>91</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>99</v>
+        <v>92</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>100</v>
+        <v>93</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>101</v>
+        <v>94</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>102</v>
+        <v>95</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>103</v>
+        <v>96</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>104</v>
+        <v>97</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>105</v>
+        <v>98</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>106</v>
+        <v>99</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>107</v>
+        <v>100</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>108</v>
+        <v>101</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>109</v>
+        <v>102</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>110</v>
+        <v>103</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>111</v>
+        <v>104</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>112</v>
+        <v>105</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>113</v>
+        <v>106</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>114</v>
+        <v>107</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>115</v>
+        <v>108</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>116</v>
+        <v>109</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>117</v>
+        <v>110</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>118</v>
+        <v>111</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>119</v>
+        <v>112</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>120</v>
+        <v>113</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>122</v>
+        <v>115</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>123</v>
+        <v>116</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>124</v>
+        <v>117</v>
       </c>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>125</v>
+        <v>118</v>
       </c>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>126</v>
+        <v>119</v>
       </c>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>127</v>
+        <v>120</v>
       </c>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>128</v>
+        <v>121</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>129</v>
+        <v>122</v>
       </c>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>130</v>
+        <v>123</v>
       </c>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
-        <v>132</v>
+        <v>125</v>
       </c>
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
-        <v>133</v>
+        <v>126</v>
       </c>
     </row>
     <row r="54" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
-        <v>134</v>
+        <v>127</v>
       </c>
     </row>
     <row r="55" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
-        <v>66</v>
+        <v>59</v>
       </c>
     </row>
     <row r="56" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
-        <v>135</v>
+        <v>128</v>
       </c>
     </row>
     <row r="57" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
-        <v>136</v>
+        <v>129</v>
       </c>
     </row>
     <row r="58" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
-        <v>137</v>
+        <v>130</v>
       </c>
     </row>
     <row r="59" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
-        <v>138</v>
+        <v>131</v>
       </c>
     </row>
     <row r="60" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
-        <v>139</v>
+        <v>132</v>
       </c>
     </row>
     <row r="61" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
-        <v>140</v>
+        <v>133</v>
       </c>
     </row>
     <row r="62" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
-        <v>141</v>
+        <v>134</v>
       </c>
     </row>
     <row r="63" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
-        <v>142</v>
+        <v>135</v>
       </c>
     </row>
     <row r="64" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
     </row>
   </sheetData>
@@ -2215,252 +2172,252 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>144</v>
+        <v>137</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>145</v>
+        <v>138</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>146</v>
+        <v>139</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>147</v>
+        <v>140</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>148</v>
+        <v>141</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>149</v>
+        <v>142</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>150</v>
+        <v>143</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>151</v>
+        <v>144</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>152</v>
+        <v>145</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>153</v>
+        <v>146</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>154</v>
+        <v>147</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>155</v>
+        <v>148</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>156</v>
+        <v>149</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>157</v>
+        <v>150</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>158</v>
+        <v>151</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>159</v>
+        <v>152</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>160</v>
+        <v>153</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>161</v>
+        <v>154</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>162</v>
+        <v>155</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>163</v>
+        <v>156</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>165</v>
+        <v>158</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>166</v>
+        <v>159</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>167</v>
+        <v>160</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>168</v>
+        <v>161</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>169</v>
+        <v>162</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>170</v>
+        <v>163</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>171</v>
+        <v>164</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>172</v>
+        <v>165</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>173</v>
+        <v>166</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>174</v>
+        <v>167</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>175</v>
+        <v>168</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>176</v>
+        <v>169</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>177</v>
+        <v>170</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>150</v>
+        <v>143</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>178</v>
+        <v>171</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>179</v>
+        <v>172</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>180</v>
+        <v>173</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>181</v>
+        <v>174</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>182</v>
+        <v>175</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>183</v>
+        <v>176</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>186</v>
+        <v>179</v>
       </c>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>187</v>
+        <v>180</v>
       </c>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>188</v>
+        <v>181</v>
       </c>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>189</v>
+        <v>182</v>
       </c>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>190</v>
+        <v>183</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>191</v>
+        <v>184</v>
       </c>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>192</v>
+        <v>185</v>
       </c>
     </row>
   </sheetData>
@@ -2480,837 +2437,837 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>193</v>
+        <v>186</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>194</v>
+        <v>187</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>195</v>
+        <v>188</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>196</v>
+        <v>189</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>197</v>
+        <v>190</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>198</v>
+        <v>191</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>199</v>
+        <v>192</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>200</v>
+        <v>193</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>201</v>
+        <v>194</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>202</v>
+        <v>195</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>203</v>
+        <v>196</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>204</v>
+        <v>197</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>205</v>
+        <v>198</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>206</v>
+        <v>199</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>207</v>
+        <v>200</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>208</v>
+        <v>201</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>209</v>
+        <v>202</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>210</v>
+        <v>203</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>211</v>
+        <v>204</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>212</v>
+        <v>205</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>213</v>
+        <v>206</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>214</v>
+        <v>207</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>215</v>
+        <v>208</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>216</v>
+        <v>209</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>217</v>
+        <v>210</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>218</v>
+        <v>211</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>219</v>
+        <v>212</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>220</v>
+        <v>213</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>221</v>
+        <v>214</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>222</v>
+        <v>215</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>223</v>
+        <v>216</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>224</v>
+        <v>217</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>225</v>
+        <v>218</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>227</v>
+        <v>220</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>228</v>
+        <v>221</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>229</v>
+        <v>222</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>230</v>
+        <v>223</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>231</v>
+        <v>224</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>232</v>
+        <v>225</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>233</v>
+        <v>226</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>234</v>
+        <v>227</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>235</v>
+        <v>228</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>236</v>
+        <v>229</v>
       </c>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>237</v>
+        <v>230</v>
       </c>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>238</v>
+        <v>231</v>
       </c>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>239</v>
+        <v>232</v>
       </c>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>240</v>
+        <v>233</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>241</v>
+        <v>234</v>
       </c>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>242</v>
+        <v>235</v>
       </c>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>243</v>
+        <v>236</v>
       </c>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
-        <v>244</v>
+        <v>237</v>
       </c>
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
-        <v>245</v>
+        <v>238</v>
       </c>
     </row>
     <row r="54" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
-        <v>246</v>
+        <v>239</v>
       </c>
     </row>
     <row r="55" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
-        <v>247</v>
+        <v>240</v>
       </c>
     </row>
     <row r="56" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
-        <v>248</v>
+        <v>241</v>
       </c>
     </row>
     <row r="57" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
-        <v>249</v>
+        <v>242</v>
       </c>
     </row>
     <row r="58" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
-        <v>250</v>
+        <v>243</v>
       </c>
     </row>
     <row r="59" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
-        <v>251</v>
+        <v>244</v>
       </c>
     </row>
     <row r="60" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
-        <v>252</v>
+        <v>245</v>
       </c>
     </row>
     <row r="61" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
-        <v>253</v>
+        <v>246</v>
       </c>
     </row>
     <row r="62" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
-        <v>254</v>
+        <v>247</v>
       </c>
     </row>
     <row r="63" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
-        <v>255</v>
+        <v>248</v>
       </c>
     </row>
     <row r="64" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
-        <v>256</v>
+        <v>249</v>
       </c>
     </row>
     <row r="65" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
-        <v>257</v>
+        <v>250</v>
       </c>
     </row>
     <row r="66" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
-        <v>258</v>
+        <v>251</v>
       </c>
     </row>
     <row r="67" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
-        <v>259</v>
+        <v>252</v>
       </c>
     </row>
     <row r="68" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
-        <v>260</v>
+        <v>253</v>
       </c>
     </row>
     <row r="69" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
-        <v>261</v>
+        <v>254</v>
       </c>
     </row>
     <row r="70" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
-        <v>262</v>
+        <v>255</v>
       </c>
     </row>
     <row r="71" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
-        <v>263</v>
+        <v>256</v>
       </c>
     </row>
     <row r="72" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
-        <v>264</v>
+        <v>257</v>
       </c>
     </row>
     <row r="73" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
-        <v>265</v>
+        <v>258</v>
       </c>
     </row>
     <row r="74" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
-        <v>266</v>
+        <v>259</v>
       </c>
     </row>
     <row r="75" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
-        <v>267</v>
+        <v>260</v>
       </c>
     </row>
     <row r="76" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
-        <v>268</v>
+        <v>261</v>
       </c>
     </row>
     <row r="77" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="78" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
-        <v>270</v>
+        <v>263</v>
       </c>
     </row>
     <row r="79" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
-        <v>271</v>
+        <v>264</v>
       </c>
     </row>
     <row r="80" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
-        <v>272</v>
+        <v>265</v>
       </c>
     </row>
     <row r="81" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
-        <v>273</v>
+        <v>266</v>
       </c>
     </row>
     <row r="82" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
-        <v>274</v>
+        <v>267</v>
       </c>
     </row>
     <row r="83" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
-        <v>275</v>
+        <v>268</v>
       </c>
     </row>
     <row r="84" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
-        <v>276</v>
+        <v>269</v>
       </c>
     </row>
     <row r="85" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
-        <v>277</v>
+        <v>270</v>
       </c>
     </row>
     <row r="86" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
-        <v>278</v>
+        <v>271</v>
       </c>
     </row>
     <row r="87" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
-        <v>279</v>
+        <v>272</v>
       </c>
     </row>
     <row r="88" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
-        <v>280</v>
+        <v>273</v>
       </c>
     </row>
     <row r="89" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
-        <v>281</v>
+        <v>274</v>
       </c>
     </row>
     <row r="90" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
-        <v>282</v>
+        <v>275</v>
       </c>
     </row>
     <row r="91" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
-        <v>283</v>
+        <v>276</v>
       </c>
     </row>
     <row r="92" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
-        <v>284</v>
+        <v>277</v>
       </c>
     </row>
     <row r="93" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
-        <v>285</v>
+        <v>278</v>
       </c>
     </row>
     <row r="94" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
-        <v>286</v>
+        <v>279</v>
       </c>
     </row>
     <row r="95" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
-        <v>287</v>
+        <v>280</v>
       </c>
     </row>
     <row r="96" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
-        <v>286</v>
+        <v>279</v>
       </c>
     </row>
     <row r="97" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
-        <v>288</v>
+        <v>281</v>
       </c>
     </row>
     <row r="98" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
-        <v>289</v>
+        <v>282</v>
       </c>
     </row>
     <row r="99" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
-        <v>290</v>
+        <v>283</v>
       </c>
     </row>
     <row r="100" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
-        <v>233</v>
+        <v>226</v>
       </c>
     </row>
     <row r="101" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
-        <v>291</v>
+        <v>284</v>
       </c>
     </row>
     <row r="102" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
-        <v>292</v>
+        <v>285</v>
       </c>
     </row>
     <row r="103" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
-        <v>293</v>
+        <v>286</v>
       </c>
     </row>
     <row r="104" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
-        <v>294</v>
+        <v>287</v>
       </c>
     </row>
     <row r="105" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
-        <v>295</v>
+        <v>288</v>
       </c>
     </row>
     <row r="106" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
-        <v>296</v>
+        <v>289</v>
       </c>
     </row>
     <row r="107" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
-        <v>297</v>
+        <v>290</v>
       </c>
     </row>
     <row r="108" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
-        <v>298</v>
+        <v>291</v>
       </c>
     </row>
     <row r="109" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A109" t="s">
-        <v>299</v>
+        <v>292</v>
       </c>
     </row>
     <row r="110" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
-        <v>300</v>
+        <v>293</v>
       </c>
     </row>
     <row r="111" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
-        <v>301</v>
+        <v>294</v>
       </c>
     </row>
     <row r="112" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
-        <v>302</v>
+        <v>295</v>
       </c>
     </row>
     <row r="113" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
-        <v>303</v>
+        <v>296</v>
       </c>
     </row>
     <row r="114" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A114" t="s">
-        <v>304</v>
+        <v>297</v>
       </c>
     </row>
     <row r="115" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A115" t="s">
-        <v>305</v>
+        <v>298</v>
       </c>
     </row>
     <row r="116" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A116" t="s">
-        <v>306</v>
+        <v>299</v>
       </c>
     </row>
     <row r="117" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A117" t="s">
-        <v>307</v>
+        <v>300</v>
       </c>
     </row>
     <row r="118" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A118" t="s">
-        <v>308</v>
+        <v>301</v>
       </c>
     </row>
     <row r="119" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A119" t="s">
-        <v>309</v>
+        <v>302</v>
       </c>
     </row>
     <row r="120" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A120" t="s">
-        <v>310</v>
+        <v>303</v>
       </c>
     </row>
     <row r="121" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A121" t="s">
-        <v>222</v>
+        <v>215</v>
       </c>
     </row>
     <row r="122" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A122" t="s">
-        <v>221</v>
+        <v>214</v>
       </c>
     </row>
     <row r="123" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A123" t="s">
-        <v>227</v>
+        <v>220</v>
       </c>
     </row>
     <row r="124" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A124" t="s">
-        <v>228</v>
+        <v>221</v>
       </c>
     </row>
     <row r="125" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A125" t="s">
-        <v>311</v>
+        <v>304</v>
       </c>
     </row>
     <row r="126" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A126" t="s">
-        <v>312</v>
+        <v>305</v>
       </c>
     </row>
     <row r="127" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A127" t="s">
-        <v>313</v>
+        <v>306</v>
       </c>
     </row>
     <row r="128" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A128" t="s">
-        <v>314</v>
+        <v>307</v>
       </c>
     </row>
     <row r="129" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A129" t="s">
-        <v>315</v>
+        <v>308</v>
       </c>
     </row>
     <row r="130" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A130" t="s">
-        <v>316</v>
+        <v>309</v>
       </c>
     </row>
     <row r="131" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A131" t="s">
-        <v>317</v>
+        <v>310</v>
       </c>
     </row>
     <row r="132" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A132" t="s">
-        <v>318</v>
+        <v>311</v>
       </c>
     </row>
     <row r="133" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A133" t="s">
-        <v>319</v>
+        <v>312</v>
       </c>
     </row>
     <row r="134" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A134" t="s">
-        <v>315</v>
+        <v>308</v>
       </c>
     </row>
     <row r="135" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A135" t="s">
-        <v>320</v>
+        <v>313</v>
       </c>
     </row>
     <row r="136" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A136" t="s">
-        <v>321</v>
+        <v>314</v>
       </c>
     </row>
     <row r="137" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A137" t="s">
-        <v>315</v>
+        <v>308</v>
       </c>
     </row>
     <row r="138" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A138" t="s">
-        <v>322</v>
+        <v>315</v>
       </c>
     </row>
     <row r="139" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A139" t="s">
-        <v>315</v>
+        <v>308</v>
       </c>
     </row>
     <row r="140" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A140" t="s">
-        <v>323</v>
+        <v>316</v>
       </c>
     </row>
     <row r="141" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A141" t="s">
-        <v>315</v>
+        <v>308</v>
       </c>
     </row>
     <row r="142" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A142" t="s">
-        <v>324</v>
+        <v>317</v>
       </c>
     </row>
     <row r="143" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A143" t="s">
-        <v>315</v>
+        <v>308</v>
       </c>
     </row>
     <row r="144" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A144" t="s">
-        <v>325</v>
+        <v>318</v>
       </c>
     </row>
     <row r="145" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A145" t="s">
-        <v>315</v>
+        <v>308</v>
       </c>
     </row>
     <row r="146" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A146" t="s">
-        <v>326</v>
+        <v>319</v>
       </c>
     </row>
     <row r="147" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A147" t="s">
-        <v>315</v>
+        <v>308</v>
       </c>
     </row>
     <row r="148" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A148" t="s">
-        <v>327</v>
+        <v>320</v>
       </c>
     </row>
     <row r="149" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A149" t="s">
-        <v>315</v>
+        <v>308</v>
       </c>
     </row>
     <row r="150" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A150" t="s">
-        <v>328</v>
+        <v>321</v>
       </c>
     </row>
     <row r="151" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A151" t="s">
-        <v>315</v>
+        <v>308</v>
       </c>
     </row>
     <row r="152" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A152" t="s">
-        <v>329</v>
+        <v>322</v>
       </c>
     </row>
     <row r="153" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A153" t="s">
-        <v>315</v>
+        <v>308</v>
       </c>
     </row>
     <row r="154" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A154" t="s">
-        <v>330</v>
+        <v>323</v>
       </c>
     </row>
     <row r="155" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A155" t="s">
-        <v>315</v>
+        <v>308</v>
       </c>
     </row>
     <row r="156" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A156" t="s">
-        <v>331</v>
+        <v>324</v>
       </c>
     </row>
     <row r="157" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A157" t="s">
-        <v>315</v>
+        <v>308</v>
       </c>
     </row>
     <row r="158" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A158" t="s">
-        <v>332</v>
+        <v>325</v>
       </c>
     </row>
     <row r="159" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A159" t="s">
-        <v>315</v>
+        <v>308</v>
       </c>
     </row>
     <row r="160" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A160" t="s">
-        <v>333</v>
+        <v>326</v>
       </c>
     </row>
     <row r="161" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A161" t="s">
-        <v>315</v>
+        <v>308</v>
       </c>
     </row>
     <row r="162" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A162" t="s">
-        <v>334</v>
+        <v>327</v>
       </c>
     </row>
     <row r="163" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A163" t="s">
-        <v>315</v>
+        <v>308</v>
       </c>
     </row>
     <row r="164" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A164" t="s">
-        <v>335</v>
+        <v>328</v>
       </c>
     </row>
     <row r="165" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A165" t="s">
-        <v>336</v>
+        <v>329</v>
       </c>
     </row>
     <row r="166" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A166" t="s">
-        <v>337</v>
+        <v>330</v>
       </c>
     </row>
     <row r="167" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A167" t="s">
-        <v>338</v>
+        <v>331</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added docs for std::quoted and std::shared_lock
</commit_message>
<xml_diff>
--- a/docs/roadmap/Roadmap - C++ New Features.xlsx
+++ b/docs/roadmap/Roadmap - C++ New Features.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\git\Cpp-Modern-Features\docs\roadmap\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git\Cpp-Modern-Features\docs\roadmap\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC09CB39-543A-4104-A4C4-CFDAA5F5F918}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90B92397-7708-4F36-BD32-1B3B120D386E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="667" uniqueCount="436">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="689" uniqueCount="436">
   <si>
     <t>Hadi Abbasi</t>
   </si>
@@ -2937,41 +2937,77 @@
       <c r="A2" t="s">
         <v>11</v>
       </c>
+      <c r="B2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>333</v>
+      </c>
+      <c r="D2" s="7" t="s">
+        <v>333</v>
+      </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>12</v>
       </c>
+      <c r="B3" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>333</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>333</v>
+      </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>13</v>
       </c>
+      <c r="B4" s="2" t="s">
+        <v>0</v>
+      </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>14</v>
       </c>
+      <c r="B5" s="2" t="s">
+        <v>0</v>
+      </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>15</v>
       </c>
+      <c r="B6" s="2" t="s">
+        <v>0</v>
+      </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>16</v>
       </c>
+      <c r="B7" s="2" t="s">
+        <v>0</v>
+      </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>17</v>
       </c>
+      <c r="B8" s="2" t="s">
+        <v>0</v>
+      </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>18</v>
       </c>
+      <c r="B9" s="2" t="s">
+        <v>0</v>
+      </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
@@ -2980,21 +3016,36 @@
       <c r="B10" s="2" t="s">
         <v>0</v>
       </c>
+      <c r="C10" s="7" t="s">
+        <v>333</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>333</v>
+      </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>20</v>
       </c>
+      <c r="B11" s="2" t="s">
+        <v>0</v>
+      </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>21</v>
       </c>
+      <c r="B12" s="2" t="s">
+        <v>0</v>
+      </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>22</v>
       </c>
+      <c r="B13" s="2" t="s">
+        <v>0</v>
+      </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
@@ -3003,20 +3054,35 @@
       <c r="B14" s="2" t="s">
         <v>0</v>
       </c>
+      <c r="C14" s="7" t="s">
+        <v>333</v>
+      </c>
+      <c r="D14" s="7" t="s">
+        <v>333</v>
+      </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>24</v>
       </c>
+      <c r="B15" s="2" t="s">
+        <v>0</v>
+      </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>25</v>
       </c>
+      <c r="B16" s="2" t="s">
+        <v>0</v>
+      </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>26</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>0</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
added docs for binary literals , relaxed constexpr
</commit_message>
<xml_diff>
--- a/docs/roadmap/Roadmap - C++ New Features.xlsx
+++ b/docs/roadmap/Roadmap - C++ New Features.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git\Cpp-Modern-Features\docs\roadmap\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90B92397-7708-4F36-BD32-1B3B120D386E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A0F5F28-0115-4016-AB4F-BB70869AA051}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="C++11" sheetId="3" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="689" uniqueCount="436">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="693" uniqueCount="436">
   <si>
     <t>Hadi Abbasi</t>
   </si>
@@ -2968,6 +2968,12 @@
       <c r="B4" s="2" t="s">
         <v>0</v>
       </c>
+      <c r="C4" s="7" t="s">
+        <v>333</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>333</v>
+      </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
@@ -2975,6 +2981,12 @@
       </c>
       <c r="B5" s="2" t="s">
         <v>0</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>333</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>333</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
added digit separator , variable templates in cpp14
</commit_message>
<xml_diff>
--- a/docs/roadmap/Roadmap - C++ New Features.xlsx
+++ b/docs/roadmap/Roadmap - C++ New Features.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git\Cpp-Modern-Features\docs\roadmap\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A0F5F28-0115-4016-AB4F-BB70869AA051}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBAFD091-ED1F-48A7-AA77-ECD9162F6608}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="693" uniqueCount="436">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="697" uniqueCount="436">
   <si>
     <t>Hadi Abbasi</t>
   </si>
@@ -2996,6 +2996,12 @@
       <c r="B6" s="2" t="s">
         <v>0</v>
       </c>
+      <c r="C6" s="7" t="s">
+        <v>333</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>333</v>
+      </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
@@ -3003,6 +3009,12 @@
       </c>
       <c r="B7" s="2" t="s">
         <v>0</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>333</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>333</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
added docs for aggregate classes with default member initializers and also for std::shared_timed_mutex in c++14
</commit_message>
<xml_diff>
--- a/docs/roadmap/Roadmap - C++ New Features.xlsx
+++ b/docs/roadmap/Roadmap - C++ New Features.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git\Cpp-Modern-Features\docs\roadmap\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF018C17-5432-440B-963F-015E9911AD09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11042FED-7A46-40D5-8EC8-ED5D22B809D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="C++11" sheetId="3" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="697" uniqueCount="436">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="707" uniqueCount="436">
   <si>
     <t>Hadi Abbasi</t>
   </si>
@@ -2381,6 +2381,12 @@
       <c r="B7" s="3" t="s">
         <v>300</v>
       </c>
+      <c r="C7" s="8" t="s">
+        <v>301</v>
+      </c>
+      <c r="D7" s="8" t="s">
+        <v>301</v>
+      </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
@@ -2389,6 +2395,12 @@
       <c r="B8" s="3" t="s">
         <v>300</v>
       </c>
+      <c r="C8" s="8" t="s">
+        <v>301</v>
+      </c>
+      <c r="D8" s="8" t="s">
+        <v>301</v>
+      </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
@@ -2396,6 +2408,12 @@
       </c>
       <c r="B9" s="3" t="s">
         <v>300</v>
+      </c>
+      <c r="C9" s="8" t="s">
+        <v>301</v>
+      </c>
+      <c r="D9" s="8" t="s">
+        <v>301</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
@@ -3024,6 +3042,12 @@
       <c r="B8" s="2" t="s">
         <v>0</v>
       </c>
+      <c r="C8" s="7" t="s">
+        <v>435</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>435</v>
+      </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
@@ -3031,6 +3055,12 @@
       </c>
       <c r="B9" s="2" t="s">
         <v>0</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>435</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>435</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
@@ -3216,8 +3246,8 @@
       <c r="B2" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="C2" s="7" t="s">
-        <v>435</v>
+      <c r="C2" s="8" t="s">
+        <v>301</v>
       </c>
       <c r="D2" s="7"/>
     </row>
@@ -3228,8 +3258,8 @@
       <c r="B3" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="C3" s="7" t="s">
-        <v>435</v>
+      <c r="C3" s="8" t="s">
+        <v>301</v>
       </c>
       <c r="D3" s="7"/>
     </row>
@@ -3240,8 +3270,8 @@
       <c r="B4" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="C4" s="7" t="s">
-        <v>435</v>
+      <c r="C4" s="8" t="s">
+        <v>301</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
@@ -3251,8 +3281,8 @@
       <c r="B5" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="C5" s="7" t="s">
-        <v>435</v>
+      <c r="C5" s="8" t="s">
+        <v>301</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
@@ -3262,8 +3292,8 @@
       <c r="B6" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="C6" s="7" t="s">
-        <v>435</v>
+      <c r="C6" s="8" t="s">
+        <v>301</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
@@ -3273,8 +3303,8 @@
       <c r="B7" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="C7" s="7" t="s">
-        <v>435</v>
+      <c r="C7" s="8" t="s">
+        <v>301</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
@@ -3284,8 +3314,8 @@
       <c r="B8" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="C8" s="7" t="s">
-        <v>435</v>
+      <c r="C8" s="8" t="s">
+        <v>301</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
@@ -3295,8 +3325,8 @@
       <c r="B9" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="C9" s="7" t="s">
-        <v>435</v>
+      <c r="C9" s="8" t="s">
+        <v>301</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
@@ -3306,8 +3336,8 @@
       <c r="B10" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="C10" s="7" t="s">
-        <v>435</v>
+      <c r="C10" s="8" t="s">
+        <v>301</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
@@ -3317,8 +3347,8 @@
       <c r="B11" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="C11" s="7" t="s">
-        <v>435</v>
+      <c r="C11" s="8" t="s">
+        <v>301</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
@@ -3328,11 +3358,11 @@
       <c r="B12" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="C12" s="7" t="s">
-        <v>435</v>
-      </c>
-      <c r="D12" s="7" t="s">
-        <v>435</v>
+      <c r="C12" s="8" t="s">
+        <v>301</v>
+      </c>
+      <c r="D12" s="8" t="s">
+        <v>301</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
@@ -3342,8 +3372,8 @@
       <c r="B13" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="C13" s="7" t="s">
-        <v>435</v>
+      <c r="C13" s="8" t="s">
+        <v>301</v>
       </c>
       <c r="D13" s="7"/>
     </row>
@@ -3354,8 +3384,8 @@
       <c r="B14" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="C14" s="7" t="s">
-        <v>435</v>
+      <c r="C14" s="8" t="s">
+        <v>301</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
@@ -3365,8 +3395,8 @@
       <c r="B15" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="C15" s="7" t="s">
-        <v>435</v>
+      <c r="C15" s="8" t="s">
+        <v>301</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.3">
@@ -3376,8 +3406,8 @@
       <c r="B16" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="C16" s="7" t="s">
-        <v>435</v>
+      <c r="C16" s="8" t="s">
+        <v>301</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
added docs for std::integer_sequence and std::index_sequence.md
</commit_message>
<xml_diff>
--- a/docs/roadmap/Roadmap - C++ New Features.xlsx
+++ b/docs/roadmap/Roadmap - C++ New Features.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git\Cpp-Modern-Features\docs\roadmap\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11042FED-7A46-40D5-8EC8-ED5D22B809D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EAB053B0-AA23-41AE-9D83-36925EF46817}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="C++11" sheetId="3" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="707" uniqueCount="436">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="711" uniqueCount="436">
   <si>
     <t>Hadi Abbasi</t>
   </si>
@@ -3084,6 +3084,12 @@
       <c r="B11" s="2" t="s">
         <v>0</v>
       </c>
+      <c r="C11" s="7" t="s">
+        <v>435</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>435</v>
+      </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
@@ -3091,6 +3097,12 @@
       </c>
       <c r="B12" s="2" t="s">
         <v>0</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>435</v>
+      </c>
+      <c r="D12" s="7" t="s">
+        <v>435</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
aded docs for std::exchange,std::tuple_element_t, std::is_final, std::make_reverse_iterator
</commit_message>
<xml_diff>
--- a/docs/roadmap/Roadmap - C++ New Features.xlsx
+++ b/docs/roadmap/Roadmap - C++ New Features.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git\Cpp-Modern-Features\docs\roadmap\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EAB053B0-AA23-41AE-9D83-36925EF46817}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A220151-80C2-4A34-B9C6-6A7FFB41097F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="711" uniqueCount="436">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="719" uniqueCount="436">
   <si>
     <t>Hadi Abbasi</t>
   </si>
@@ -3112,6 +3112,12 @@
       <c r="B13" s="2" t="s">
         <v>0</v>
       </c>
+      <c r="C13" s="7" t="s">
+        <v>435</v>
+      </c>
+      <c r="D13" s="7" t="s">
+        <v>435</v>
+      </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
@@ -3134,6 +3140,12 @@
       <c r="B15" s="2" t="s">
         <v>0</v>
       </c>
+      <c r="C15" s="7" t="s">
+        <v>435</v>
+      </c>
+      <c r="D15" s="7" t="s">
+        <v>435</v>
+      </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
@@ -3142,6 +3154,12 @@
       <c r="B16" s="2" t="s">
         <v>0</v>
       </c>
+      <c r="C16" s="7" t="s">
+        <v>435</v>
+      </c>
+      <c r="D16" s="7" t="s">
+        <v>435</v>
+      </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
@@ -3149,6 +3167,12 @@
       </c>
       <c r="B17" s="2" t="s">
         <v>0</v>
+      </c>
+      <c r="C17" s="7" t="s">
+        <v>435</v>
+      </c>
+      <c r="D17" s="7" t="s">
+        <v>435</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
added documents for [[no_unique_address]] and char8_t in C++20
</commit_message>
<xml_diff>
--- a/docs/roadmap/Roadmap - C++ New Features.xlsx
+++ b/docs/roadmap/Roadmap - C++ New Features.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git\Cpp-Modern-Features\docs\roadmap\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A220151-80C2-4A34-B9C6-6A7FFB41097F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77953D09-887A-4160-AF38-593DE2E4B486}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="C++11" sheetId="3" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="719" uniqueCount="436">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="762" uniqueCount="436">
   <si>
     <t>Hadi Abbasi</t>
   </si>
@@ -3648,12 +3648,8 @@
       <c r="B3" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="7" t="s">
-        <v>435</v>
-      </c>
-      <c r="D3" s="7" t="s">
-        <v>435</v>
-      </c>
+      <c r="C3" s="7"/>
+      <c r="D3" s="7"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
@@ -3673,6 +3669,9 @@
       <c r="A5" t="s">
         <v>70</v>
       </c>
+      <c r="B5" s="3" t="s">
+        <v>0</v>
+      </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
@@ -3729,264 +3728,396 @@
         <v>81</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B17" s="3" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B18" s="3" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>84</v>
       </c>
-    </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B19" s="3" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>85</v>
       </c>
-    </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B20" s="3" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>86</v>
       </c>
-    </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B21" s="3" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>87</v>
       </c>
-    </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B22" s="3" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B23" s="3" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>89</v>
       </c>
-    </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B24" s="3" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>90</v>
       </c>
-    </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B25" s="3" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>91</v>
       </c>
-    </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B26" s="3" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>92</v>
       </c>
-    </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B27" s="3" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>93</v>
       </c>
-    </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B28" s="3" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B29" s="3" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B30" s="3" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B31" s="3" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>97</v>
       </c>
-    </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B32" s="3" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B33" s="3" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>100</v>
       </c>
-    </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B35" s="3" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B37" s="3" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B38" s="3" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>105</v>
       </c>
-    </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B40" s="3" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>106</v>
       </c>
-    </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B41" s="3" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="43" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>108</v>
       </c>
-    </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B43" s="3" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="46" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="47" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="48" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B48" s="3" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>114</v>
       </c>
-    </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B49" s="3" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>115</v>
       </c>
-    </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B50" s="3" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>116</v>
       </c>
-    </row>
-    <row r="52" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B51" s="3" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="53" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="54" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="55" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="56" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>121</v>
       </c>
-    </row>
-    <row r="57" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B56" s="3" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="58" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B57" s="3" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>123</v>
       </c>
-    </row>
-    <row r="59" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B58" s="3" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="60" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B59" s="3" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>124</v>
       </c>
-    </row>
-    <row r="61" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B60" s="3" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>125</v>
       </c>
-    </row>
-    <row r="62" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B61" s="3" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>126</v>
       </c>
-    </row>
-    <row r="63" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B62" s="3" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>127</v>
       </c>
-    </row>
-    <row r="64" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B63" s="3" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="65" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B64" s="3" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>129</v>
       </c>
-    </row>
-    <row r="66" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B65" s="3" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>130</v>
       </c>
-    </row>
-    <row r="67" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B66" s="3" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>131</v>
       </c>
-    </row>
-    <row r="68" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B67" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="C67" s="7" t="s">
+        <v>435</v>
+      </c>
+      <c r="D67" s="7" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>132</v>
+      </c>
+      <c r="B68" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="C68" s="7" t="s">
+        <v>435</v>
+      </c>
+      <c r="D68" s="7" t="s">
+        <v>435</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added c++20 features (constexpr, concepts_requires_constraints_type_traits, std::span , spaceship operator)
</commit_message>
<xml_diff>
--- a/docs/roadmap/Roadmap - C++ New Features.xlsx
+++ b/docs/roadmap/Roadmap - C++ New Features.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git\Cpp-Modern-Features\docs\roadmap\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77953D09-887A-4160-AF38-593DE2E4B486}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2635B9DF-63C8-4C39-A3CB-328679D12CB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="C++11" sheetId="3" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="762" uniqueCount="436">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="735" uniqueCount="413">
   <si>
     <t>Hadi Abbasi</t>
   </si>
@@ -246,88 +246,7 @@
     <t>Three-way comparison / Spaceship Operator &lt;=&gt;</t>
   </si>
   <si>
-    <t>Concepts</t>
-  </si>
-  <si>
-    <t>requires</t>
-  </si>
-  <si>
-    <t>Constraints</t>
-  </si>
-  <si>
     <t>Abbreviated Function Templates</t>
-  </si>
-  <si>
-    <t>Modules</t>
-  </si>
-  <si>
-    <t>import</t>
-  </si>
-  <si>
-    <t>export module</t>
-  </si>
-  <si>
-    <t>Coroutines</t>
-  </si>
-  <si>
-    <t>co_await</t>
-  </si>
-  <si>
-    <t>co_yield</t>
-  </si>
-  <si>
-    <t>co_return</t>
-  </si>
-  <si>
-    <t>Ranges</t>
-  </si>
-  <si>
-    <t>std::ranges</t>
-  </si>
-  <si>
-    <t>std::views</t>
-  </si>
-  <si>
-    <t>Range Views</t>
-  </si>
-  <si>
-    <t>views::filter</t>
-  </si>
-  <si>
-    <t>views::transform</t>
-  </si>
-  <si>
-    <t>views::take</t>
-  </si>
-  <si>
-    <t>views::drop</t>
-  </si>
-  <si>
-    <t>views::reverse</t>
-  </si>
-  <si>
-    <t>views::keys</t>
-  </si>
-  <si>
-    <t>views::values</t>
-  </si>
-  <si>
-    <t>views::iota</t>
-  </si>
-  <si>
-    <t>views::join</t>
-  </si>
-  <si>
-    <t>Range Algorithms</t>
-  </si>
-  <si>
-    <t>ranges::sort</t>
-  </si>
-  <si>
-    <t>ranges::find</t>
-  </si>
-  <si>
-    <t>ranges::for_each</t>
   </si>
   <si>
     <t>Designated Initializers</t>
@@ -1860,6 +1779,18 @@
   </si>
   <si>
     <t>Done (Review Required)</t>
+  </si>
+  <si>
+    <t>Concepts , requires , Constraints</t>
+  </si>
+  <si>
+    <t>Modules + import + export module</t>
+  </si>
+  <si>
+    <t>Coroutines + co_await + co_yield + co_return</t>
+  </si>
+  <si>
+    <t>std::ranges + std::views + Range Views + views::filter + views::transform + views::take + views::drop +views::reverse +  views::keys + views::values + views::iota + views::join + Range Algorithms + ranges::sort + ranges::find + ranges::for_each</t>
   </si>
 </sst>
 </file>
@@ -2292,16 +2223,16 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
-        <v>295</v>
+        <v>268</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>298</v>
+        <v>271</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>296</v>
+        <v>269</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>297</v>
+        <v>270</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
@@ -2312,10 +2243,10 @@
         <v>0</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>435</v>
+        <v>408</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>435</v>
+        <v>408</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
@@ -2326,10 +2257,10 @@
         <v>0</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>435</v>
+        <v>408</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>435</v>
+        <v>408</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
@@ -2340,10 +2271,10 @@
         <v>0</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>435</v>
+        <v>408</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>435</v>
+        <v>408</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
@@ -2354,10 +2285,10 @@
         <v>0</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>435</v>
+        <v>408</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>435</v>
+        <v>408</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
@@ -2368,38 +2299,38 @@
         <v>0</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>435</v>
+        <v>408</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>435</v>
+        <v>408</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>293</v>
+        <v>266</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>300</v>
+        <v>273</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>301</v>
+        <v>274</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>301</v>
+        <v>274</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>294</v>
+        <v>267</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>300</v>
+        <v>273</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>301</v>
+        <v>274</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>301</v>
+        <v>274</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
@@ -2407,13 +2338,13 @@
         <v>5</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>300</v>
+        <v>273</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>301</v>
+        <v>274</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>301</v>
+        <v>274</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
@@ -2424,10 +2355,10 @@
         <v>0</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>435</v>
+        <v>408</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>435</v>
+        <v>408</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
@@ -2438,10 +2369,10 @@
         <v>0</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>435</v>
+        <v>408</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>435</v>
+        <v>408</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
@@ -2452,10 +2383,10 @@
         <v>0</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>435</v>
+        <v>408</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>435</v>
+        <v>408</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
@@ -2466,458 +2397,458 @@
         <v>0</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>435</v>
+        <v>408</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>435</v>
+        <v>408</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>299</v>
+        <v>272</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>300</v>
+        <v>273</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>301</v>
+        <v>274</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>301</v>
+        <v>274</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>302</v>
+        <v>275</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>300</v>
+        <v>273</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>301</v>
+        <v>274</v>
       </c>
       <c r="D15" s="8" t="s">
-        <v>301</v>
+        <v>274</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>303</v>
+        <v>276</v>
       </c>
       <c r="B16" s="3" t="s">
         <v>0</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>301</v>
+        <v>274</v>
       </c>
       <c r="D16" s="8" t="s">
-        <v>301</v>
+        <v>274</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>313</v>
+        <v>286</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>300</v>
+        <v>273</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>301</v>
+        <v>274</v>
       </c>
       <c r="D17" s="8" t="s">
-        <v>301</v>
+        <v>274</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>304</v>
+        <v>277</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>300</v>
+        <v>273</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>301</v>
+        <v>274</v>
       </c>
       <c r="D18" s="8" t="s">
-        <v>301</v>
+        <v>274</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>305</v>
+        <v>278</v>
       </c>
       <c r="B19" s="3" t="s">
         <v>0</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>435</v>
+        <v>408</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>435</v>
+        <v>408</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>306</v>
+        <v>279</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>300</v>
+        <v>273</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>301</v>
+        <v>274</v>
       </c>
       <c r="D20" s="8" t="s">
-        <v>301</v>
+        <v>274</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>307</v>
+        <v>280</v>
       </c>
       <c r="B21" s="3" t="s">
         <v>0</v>
       </c>
       <c r="C21" s="7" t="s">
-        <v>435</v>
+        <v>408</v>
       </c>
       <c r="D21" s="7" t="s">
-        <v>435</v>
+        <v>408</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>308</v>
+        <v>281</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>300</v>
+        <v>273</v>
       </c>
       <c r="C22" s="8" t="s">
-        <v>301</v>
+        <v>274</v>
       </c>
       <c r="D22" s="8" t="s">
-        <v>301</v>
+        <v>274</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>309</v>
+        <v>282</v>
       </c>
       <c r="B23" s="3" t="s">
         <v>0</v>
       </c>
       <c r="C23" s="7" t="s">
-        <v>435</v>
+        <v>408</v>
       </c>
       <c r="D23" s="7" t="s">
-        <v>435</v>
+        <v>408</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>310</v>
+        <v>283</v>
       </c>
       <c r="B24" s="3" t="s">
         <v>0</v>
       </c>
       <c r="C24" s="7" t="s">
-        <v>435</v>
+        <v>408</v>
       </c>
       <c r="D24" s="7" t="s">
-        <v>435</v>
+        <v>408</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>312</v>
+        <v>285</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>300</v>
+        <v>273</v>
       </c>
       <c r="C25" s="8" t="s">
-        <v>301</v>
+        <v>274</v>
       </c>
       <c r="D25" s="8" t="s">
-        <v>301</v>
+        <v>274</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>311</v>
+        <v>284</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>300</v>
+        <v>273</v>
       </c>
       <c r="C26" s="8" t="s">
-        <v>301</v>
+        <v>274</v>
       </c>
       <c r="D26" s="8" t="s">
-        <v>301</v>
+        <v>274</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>314</v>
+        <v>287</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>300</v>
+        <v>273</v>
       </c>
       <c r="C27" s="8" t="s">
-        <v>301</v>
+        <v>274</v>
       </c>
       <c r="D27" s="8" t="s">
-        <v>301</v>
+        <v>274</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>315</v>
+        <v>288</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>300</v>
+        <v>273</v>
       </c>
       <c r="C28" s="8" t="s">
-        <v>301</v>
+        <v>274</v>
       </c>
       <c r="D28" s="8" t="s">
-        <v>301</v>
+        <v>274</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>316</v>
+        <v>289</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>300</v>
+        <v>273</v>
       </c>
       <c r="C29" s="8" t="s">
-        <v>301</v>
+        <v>274</v>
       </c>
       <c r="D29" s="8" t="s">
-        <v>301</v>
+        <v>274</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>317</v>
+        <v>290</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>300</v>
+        <v>273</v>
       </c>
       <c r="C30" s="8" t="s">
-        <v>301</v>
+        <v>274</v>
       </c>
       <c r="D30" s="8" t="s">
-        <v>301</v>
+        <v>274</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>332</v>
+        <v>305</v>
       </c>
       <c r="B31" s="3" t="s">
         <v>0</v>
       </c>
       <c r="C31" s="7" t="s">
-        <v>435</v>
+        <v>408</v>
       </c>
       <c r="D31" s="7" t="s">
-        <v>435</v>
+        <v>408</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>318</v>
+        <v>291</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>300</v>
+        <v>273</v>
       </c>
       <c r="C32" s="8" t="s">
-        <v>301</v>
+        <v>274</v>
       </c>
       <c r="D32" s="8" t="s">
-        <v>301</v>
+        <v>274</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>319</v>
+        <v>292</v>
       </c>
       <c r="B33" s="3" t="s">
         <v>0</v>
       </c>
       <c r="C33" s="7" t="s">
-        <v>435</v>
+        <v>408</v>
       </c>
       <c r="D33" s="7" t="s">
-        <v>435</v>
+        <v>408</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>320</v>
+        <v>293</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>300</v>
+        <v>273</v>
       </c>
       <c r="C34" s="8" t="s">
-        <v>301</v>
+        <v>274</v>
       </c>
       <c r="D34" s="8" t="s">
-        <v>301</v>
+        <v>274</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>321</v>
+        <v>294</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>300</v>
+        <v>273</v>
       </c>
       <c r="C35" s="8" t="s">
-        <v>301</v>
+        <v>274</v>
       </c>
       <c r="D35" s="8" t="s">
-        <v>301</v>
+        <v>274</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>322</v>
+        <v>295</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>300</v>
+        <v>273</v>
       </c>
       <c r="C36" s="8" t="s">
-        <v>301</v>
+        <v>274</v>
       </c>
       <c r="D36" s="8" t="s">
-        <v>301</v>
+        <v>274</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>323</v>
+        <v>296</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>300</v>
+        <v>273</v>
       </c>
       <c r="C37" s="8" t="s">
-        <v>301</v>
+        <v>274</v>
       </c>
       <c r="D37" s="8" t="s">
-        <v>301</v>
+        <v>274</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>324</v>
+        <v>297</v>
       </c>
       <c r="B38" s="3" t="s">
         <v>0</v>
       </c>
       <c r="C38" s="8" t="s">
-        <v>301</v>
+        <v>274</v>
       </c>
       <c r="D38" s="8" t="s">
-        <v>301</v>
+        <v>274</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>325</v>
+        <v>298</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>300</v>
+        <v>273</v>
       </c>
       <c r="C39" s="8" t="s">
-        <v>301</v>
+        <v>274</v>
       </c>
       <c r="D39" s="8" t="s">
-        <v>301</v>
+        <v>274</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>326</v>
+        <v>299</v>
       </c>
       <c r="B40" s="3" t="s">
         <v>0</v>
       </c>
       <c r="C40" s="8" t="s">
-        <v>301</v>
+        <v>274</v>
       </c>
       <c r="D40" s="8" t="s">
-        <v>301</v>
+        <v>274</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>327</v>
+        <v>300</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>300</v>
+        <v>273</v>
       </c>
       <c r="C41" s="8" t="s">
-        <v>301</v>
+        <v>274</v>
       </c>
       <c r="D41" s="8" t="s">
-        <v>301</v>
+        <v>274</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>328</v>
+        <v>301</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>300</v>
+        <v>273</v>
       </c>
       <c r="C42" s="8" t="s">
-        <v>301</v>
+        <v>274</v>
       </c>
       <c r="D42" s="8" t="s">
-        <v>301</v>
+        <v>274</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>329</v>
+        <v>302</v>
       </c>
       <c r="B43" s="3" t="s">
         <v>0</v>
       </c>
       <c r="C43" s="8" t="s">
-        <v>301</v>
+        <v>274</v>
       </c>
       <c r="D43" s="8" t="s">
-        <v>301</v>
+        <v>274</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>330</v>
+        <v>303</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>300</v>
+        <v>273</v>
       </c>
       <c r="C44" s="8" t="s">
-        <v>301</v>
+        <v>274</v>
       </c>
       <c r="D44" s="8" t="s">
-        <v>301</v>
+        <v>274</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>331</v>
+        <v>304</v>
       </c>
       <c r="B45" s="3" t="s">
         <v>0</v>
       </c>
       <c r="C45" s="8" t="s">
-        <v>301</v>
+        <v>274</v>
       </c>
       <c r="D45" s="8" t="s">
-        <v>301</v>
+        <v>274</v>
       </c>
     </row>
   </sheetData>
@@ -2939,16 +2870,16 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
-        <v>295</v>
+        <v>268</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>298</v>
+        <v>271</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>296</v>
+        <v>269</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>297</v>
+        <v>270</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
@@ -2959,10 +2890,10 @@
         <v>0</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>435</v>
+        <v>408</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>435</v>
+        <v>408</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
@@ -2973,10 +2904,10 @@
         <v>0</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>435</v>
+        <v>408</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>435</v>
+        <v>408</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
@@ -2987,10 +2918,10 @@
         <v>0</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>435</v>
+        <v>408</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>435</v>
+        <v>408</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
@@ -3001,10 +2932,10 @@
         <v>0</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>435</v>
+        <v>408</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>435</v>
+        <v>408</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
@@ -3015,10 +2946,10 @@
         <v>0</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>435</v>
+        <v>408</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>435</v>
+        <v>408</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
@@ -3029,10 +2960,10 @@
         <v>0</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>435</v>
+        <v>408</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>435</v>
+        <v>408</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
@@ -3043,10 +2974,10 @@
         <v>0</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>435</v>
+        <v>408</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>435</v>
+        <v>408</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
@@ -3057,10 +2988,10 @@
         <v>0</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>435</v>
+        <v>408</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>435</v>
+        <v>408</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
@@ -3071,10 +3002,10 @@
         <v>0</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>435</v>
+        <v>408</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>435</v>
+        <v>408</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
@@ -3085,10 +3016,10 @@
         <v>0</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>435</v>
+        <v>408</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>435</v>
+        <v>408</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
@@ -3099,10 +3030,10 @@
         <v>0</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>435</v>
+        <v>408</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>435</v>
+        <v>408</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
@@ -3113,10 +3044,10 @@
         <v>0</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>435</v>
+        <v>408</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>435</v>
+        <v>408</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
@@ -3127,10 +3058,10 @@
         <v>0</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>435</v>
+        <v>408</v>
       </c>
       <c r="D14" s="7" t="s">
-        <v>435</v>
+        <v>408</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
@@ -3141,10 +3072,10 @@
         <v>0</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>435</v>
+        <v>408</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>435</v>
+        <v>408</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.3">
@@ -3155,10 +3086,10 @@
         <v>0</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>435</v>
+        <v>408</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>435</v>
+        <v>408</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.3">
@@ -3169,80 +3100,80 @@
         <v>0</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>435</v>
+        <v>408</v>
       </c>
       <c r="D17" s="7" t="s">
-        <v>435</v>
+        <v>408</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>425</v>
+        <v>398</v>
       </c>
       <c r="B18" s="2" t="s">
         <v>0</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>435</v>
+        <v>408</v>
       </c>
       <c r="D18" s="7" t="s">
-        <v>435</v>
+        <v>408</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>426</v>
+        <v>399</v>
       </c>
       <c r="B19" s="2" t="s">
         <v>0</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>435</v>
+        <v>408</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>435</v>
+        <v>408</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>427</v>
+        <v>400</v>
       </c>
       <c r="B20" s="2" t="s">
         <v>0</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>435</v>
+        <v>408</v>
       </c>
       <c r="D20" s="7" t="s">
-        <v>435</v>
+        <v>408</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>428</v>
+        <v>401</v>
       </c>
       <c r="B21" s="2" t="s">
         <v>0</v>
       </c>
       <c r="C21" s="7" t="s">
-        <v>435</v>
+        <v>408</v>
       </c>
       <c r="D21" s="7" t="s">
-        <v>435</v>
+        <v>408</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>429</v>
+        <v>402</v>
       </c>
       <c r="B22" s="2" t="s">
         <v>0</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>435</v>
+        <v>408</v>
       </c>
       <c r="D22" s="7" t="s">
-        <v>435</v>
+        <v>408</v>
       </c>
     </row>
   </sheetData>
@@ -3263,16 +3194,16 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
-        <v>295</v>
+        <v>268</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>298</v>
+        <v>271</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>296</v>
+        <v>269</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>297</v>
+        <v>270</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
@@ -3283,7 +3214,7 @@
         <v>36</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>301</v>
+        <v>274</v>
       </c>
       <c r="D2" s="7"/>
     </row>
@@ -3295,7 +3226,7 @@
         <v>36</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>301</v>
+        <v>274</v>
       </c>
       <c r="D3" s="7"/>
     </row>
@@ -3307,7 +3238,7 @@
         <v>36</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>301</v>
+        <v>274</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
@@ -3318,7 +3249,7 @@
         <v>36</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>301</v>
+        <v>274</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
@@ -3329,18 +3260,18 @@
         <v>36</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>301</v>
+        <v>274</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>431</v>
+        <v>404</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>36</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>301</v>
+        <v>274</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
@@ -3351,7 +3282,7 @@
         <v>36</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>301</v>
+        <v>274</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
@@ -3362,7 +3293,7 @@
         <v>36</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>301</v>
+        <v>274</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
@@ -3373,7 +3304,7 @@
         <v>36</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>301</v>
+        <v>274</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
@@ -3384,21 +3315,21 @@
         <v>36</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>301</v>
+        <v>274</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>430</v>
+        <v>403</v>
       </c>
       <c r="B12" s="3" t="s">
         <v>36</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>301</v>
+        <v>274</v>
       </c>
       <c r="D12" s="8" t="s">
-        <v>301</v>
+        <v>274</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
@@ -3409,7 +3340,7 @@
         <v>36</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>301</v>
+        <v>274</v>
       </c>
       <c r="D13" s="7"/>
     </row>
@@ -3421,7 +3352,7 @@
         <v>36</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>301</v>
+        <v>274</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
@@ -3432,18 +3363,18 @@
         <v>36</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>301</v>
+        <v>274</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>432</v>
+        <v>405</v>
       </c>
       <c r="B16" s="3" t="s">
         <v>36</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>301</v>
+        <v>274</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.3">
@@ -3603,7 +3534,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C76AFCE9-552A-4DD6-A175-0A6DA510C2C3}">
-  <dimension ref="A1:M68"/>
+  <dimension ref="A1:M44"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="55.5546875" customWidth="1"/>
@@ -3615,54 +3546,58 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
-        <v>295</v>
+        <v>268</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>298</v>
+        <v>271</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>296</v>
+        <v>269</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>297</v>
+        <v>270</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>433</v>
+        <v>406</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>0</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>435</v>
+        <v>408</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>435</v>
+        <v>408</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>305</v>
+        <v>73</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="7"/>
-      <c r="D3" s="7"/>
+      <c r="C3" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>408</v>
+      </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>434</v>
+        <v>407</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>0</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>435</v>
+        <v>408</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>435</v>
+        <v>408</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
@@ -3672,65 +3607,128 @@
       <c r="B5" s="3" t="s">
         <v>0</v>
       </c>
+      <c r="C5" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>408</v>
+      </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>71</v>
+        <v>409</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>408</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>72</v>
+        <v>78</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>408</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>73</v>
+        <v>104</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>408</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>74</v>
+        <v>105</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>408</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>75</v>
+        <v>71</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>76</v>
+        <v>410</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>77</v>
+        <v>411</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>78</v>
+        <v>412</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>79</v>
+        <v>75</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>80</v>
+        <v>76</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>81</v>
+        <v>77</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>0</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="B17" s="3" t="s">
         <v>0</v>
@@ -3738,7 +3736,7 @@
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="B18" s="3" t="s">
         <v>0</v>
@@ -3746,7 +3744,7 @@
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="B19" s="3" t="s">
         <v>0</v>
@@ -3754,7 +3752,7 @@
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B20" s="3" t="s">
         <v>0</v>
@@ -3762,7 +3760,7 @@
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B21" s="3" t="s">
         <v>0</v>
@@ -3770,7 +3768,7 @@
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B22" s="3" t="s">
         <v>0</v>
@@ -3778,7 +3776,7 @@
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B23" s="3" t="s">
         <v>0</v>
@@ -3786,7 +3784,7 @@
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="B24" s="3" t="s">
         <v>0</v>
@@ -3794,7 +3792,7 @@
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="B25" s="3" t="s">
         <v>0</v>
@@ -3802,7 +3800,7 @@
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="B26" s="3" t="s">
         <v>0</v>
@@ -3810,7 +3808,7 @@
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>92</v>
+        <v>55</v>
       </c>
       <c r="B27" s="3" t="s">
         <v>0</v>
@@ -3818,7 +3816,7 @@
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="B28" s="3" t="s">
         <v>0</v>
@@ -3826,7 +3824,7 @@
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="B29" s="3" t="s">
         <v>0</v>
@@ -3834,7 +3832,7 @@
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="B30" s="3" t="s">
         <v>0</v>
@@ -3842,7 +3840,7 @@
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="B31" s="3" t="s">
         <v>0</v>
@@ -3850,7 +3848,7 @@
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="B32" s="3" t="s">
         <v>0</v>
@@ -3858,7 +3856,7 @@
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="B33" s="3" t="s">
         <v>0</v>
@@ -3866,258 +3864,60 @@
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>99</v>
+        <v>103</v>
+      </c>
+      <c r="B34" s="3" t="s">
+        <v>0</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>100</v>
-      </c>
-      <c r="B35" s="3" t="s">
-        <v>0</v>
+        <v>90</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>101</v>
+        <v>91</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>102</v>
-      </c>
-      <c r="B37" s="3" t="s">
-        <v>0</v>
+        <v>92</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>103</v>
-      </c>
-      <c r="B38" s="3" t="s">
-        <v>0</v>
+        <v>93</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>104</v>
+        <v>72</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>105</v>
-      </c>
-      <c r="B40" s="3" t="s">
-        <v>0</v>
+        <v>74</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>106</v>
-      </c>
-      <c r="B41" s="3" t="s">
-        <v>0</v>
+        <v>82</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>107</v>
+        <v>83</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>108</v>
-      </c>
-      <c r="B43" s="3" t="s">
-        <v>0</v>
+        <v>84</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A45" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A46" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A47" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A48" t="s">
-        <v>113</v>
-      </c>
-      <c r="B48" s="3" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A49" t="s">
-        <v>114</v>
-      </c>
-      <c r="B49" s="3" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A50" t="s">
-        <v>115</v>
-      </c>
-      <c r="B50" s="3" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A51" t="s">
-        <v>116</v>
-      </c>
-      <c r="B51" s="3" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A52" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A53" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A54" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A55" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A56" t="s">
-        <v>121</v>
-      </c>
-      <c r="B56" s="3" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A57" t="s">
-        <v>122</v>
-      </c>
-      <c r="B57" s="3" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A58" t="s">
-        <v>123</v>
-      </c>
-      <c r="B58" s="3" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A59" t="s">
-        <v>55</v>
-      </c>
-      <c r="B59" s="3" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A60" t="s">
-        <v>124</v>
-      </c>
-      <c r="B60" s="3" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A61" t="s">
-        <v>125</v>
-      </c>
-      <c r="B61" s="3" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A62" t="s">
-        <v>126</v>
-      </c>
-      <c r="B62" s="3" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A63" t="s">
-        <v>127</v>
-      </c>
-      <c r="B63" s="3" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="64" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A64" t="s">
-        <v>128</v>
-      </c>
-      <c r="B64" s="3" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A65" t="s">
-        <v>129</v>
-      </c>
-      <c r="B65" s="3" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A66" t="s">
-        <v>130</v>
-      </c>
-      <c r="B66" s="3" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A67" t="s">
-        <v>131</v>
-      </c>
-      <c r="B67" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="C67" s="7" t="s">
-        <v>435</v>
-      </c>
-      <c r="D67" s="7" t="s">
-        <v>435</v>
-      </c>
-    </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A68" t="s">
-        <v>132</v>
-      </c>
-      <c r="B68" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="C68" s="7" t="s">
-        <v>435</v>
-      </c>
-      <c r="D68" s="7" t="s">
-        <v>435</v>
+        <v>85</v>
       </c>
     </row>
   </sheetData>
@@ -4139,266 +3939,266 @@
   <sheetData>
     <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
-        <v>295</v>
+        <v>268</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>298</v>
+        <v>271</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>296</v>
+        <v>269</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>297</v>
+        <v>270</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>133</v>
+        <v>106</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>134</v>
+        <v>107</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>135</v>
+        <v>108</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>136</v>
+        <v>109</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>137</v>
+        <v>110</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>138</v>
+        <v>111</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>139</v>
+        <v>112</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>140</v>
+        <v>113</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>141</v>
+        <v>114</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>142</v>
+        <v>115</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>143</v>
+        <v>116</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>144</v>
+        <v>117</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>145</v>
+        <v>118</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>146</v>
+        <v>119</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>147</v>
+        <v>120</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>148</v>
+        <v>121</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>149</v>
+        <v>122</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>150</v>
+        <v>123</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>151</v>
+        <v>124</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>152</v>
+        <v>125</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>153</v>
+        <v>126</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>154</v>
+        <v>127</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>155</v>
+        <v>128</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>156</v>
+        <v>129</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>157</v>
+        <v>130</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>158</v>
+        <v>131</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>159</v>
+        <v>132</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>160</v>
+        <v>133</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>161</v>
+        <v>134</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>162</v>
+        <v>135</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>163</v>
+        <v>136</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>164</v>
+        <v>137</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>165</v>
+        <v>138</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>166</v>
+        <v>139</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>139</v>
+        <v>112</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>167</v>
+        <v>140</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>168</v>
+        <v>141</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>169</v>
+        <v>142</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>170</v>
+        <v>143</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>171</v>
+        <v>144</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>172</v>
+        <v>145</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>173</v>
+        <v>146</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>174</v>
+        <v>147</v>
       </c>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>175</v>
+        <v>148</v>
       </c>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>176</v>
+        <v>149</v>
       </c>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>177</v>
+        <v>150</v>
       </c>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>178</v>
+        <v>151</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>179</v>
+        <v>152</v>
       </c>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>180</v>
+        <v>153</v>
       </c>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>181</v>
+        <v>154</v>
       </c>
     </row>
   </sheetData>
@@ -4420,626 +4220,626 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
-        <v>295</v>
+        <v>268</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>298</v>
+        <v>271</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>296</v>
+        <v>269</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>297</v>
+        <v>270</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>182</v>
+        <v>155</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>183</v>
+        <v>156</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>184</v>
+        <v>157</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>185</v>
+        <v>158</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>186</v>
+        <v>159</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>187</v>
+        <v>160</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>188</v>
+        <v>161</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>189</v>
+        <v>162</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>190</v>
+        <v>163</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>191</v>
+        <v>164</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>192</v>
+        <v>165</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>193</v>
+        <v>166</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>194</v>
+        <v>167</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>195</v>
+        <v>168</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>196</v>
+        <v>169</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>197</v>
+        <v>170</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>198</v>
+        <v>171</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>199</v>
+        <v>172</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>200</v>
+        <v>173</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>201</v>
+        <v>174</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>202</v>
+        <v>175</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>203</v>
+        <v>176</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>204</v>
+        <v>177</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>205</v>
+        <v>178</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>206</v>
+        <v>179</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>207</v>
+        <v>180</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>208</v>
+        <v>181</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>209</v>
+        <v>182</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>210</v>
+        <v>183</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>211</v>
+        <v>184</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>212</v>
+        <v>185</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>213</v>
+        <v>186</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>214</v>
+        <v>187</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>215</v>
+        <v>188</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>216</v>
+        <v>189</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>217</v>
+        <v>190</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>218</v>
+        <v>191</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>219</v>
+        <v>192</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>220</v>
+        <v>193</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>221</v>
+        <v>194</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>222</v>
+        <v>195</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>223</v>
+        <v>196</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>224</v>
+        <v>197</v>
       </c>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>225</v>
+        <v>198</v>
       </c>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>339</v>
+        <v>312</v>
       </c>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>226</v>
+        <v>199</v>
       </c>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>338</v>
+        <v>311</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>227</v>
+        <v>200</v>
       </c>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>337</v>
+        <v>310</v>
       </c>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>336</v>
+        <v>309</v>
       </c>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
-        <v>335</v>
+        <v>308</v>
       </c>
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
-        <v>228</v>
+        <v>201</v>
       </c>
     </row>
     <row r="54" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
-        <v>229</v>
+        <v>202</v>
       </c>
     </row>
     <row r="55" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
-        <v>230</v>
+        <v>203</v>
       </c>
     </row>
     <row r="56" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
-        <v>231</v>
+        <v>204</v>
       </c>
     </row>
     <row r="57" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
-        <v>232</v>
+        <v>205</v>
       </c>
     </row>
     <row r="58" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
-        <v>233</v>
+        <v>206</v>
       </c>
     </row>
     <row r="59" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
-        <v>234</v>
+        <v>207</v>
       </c>
     </row>
     <row r="60" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
-        <v>235</v>
+        <v>208</v>
       </c>
     </row>
     <row r="61" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
-        <v>236</v>
+        <v>209</v>
       </c>
     </row>
     <row r="62" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
-        <v>237</v>
+        <v>210</v>
       </c>
     </row>
     <row r="63" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
-        <v>238</v>
+        <v>211</v>
       </c>
     </row>
     <row r="64" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
-        <v>239</v>
+        <v>212</v>
       </c>
     </row>
     <row r="65" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
-        <v>240</v>
+        <v>213</v>
       </c>
     </row>
     <row r="66" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
-        <v>241</v>
+        <v>214</v>
       </c>
     </row>
     <row r="67" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
-        <v>242</v>
+        <v>215</v>
       </c>
     </row>
     <row r="68" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
-        <v>333</v>
+        <v>306</v>
       </c>
     </row>
     <row r="69" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
-        <v>243</v>
+        <v>216</v>
       </c>
     </row>
     <row r="70" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
-        <v>334</v>
+        <v>307</v>
       </c>
     </row>
     <row r="71" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
-        <v>244</v>
+        <v>217</v>
       </c>
     </row>
     <row r="72" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
-        <v>245</v>
+        <v>218</v>
       </c>
     </row>
     <row r="73" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
-        <v>246</v>
+        <v>219</v>
       </c>
     </row>
     <row r="74" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
-        <v>247</v>
+        <v>220</v>
       </c>
     </row>
     <row r="75" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
-        <v>248</v>
+        <v>221</v>
       </c>
     </row>
     <row r="76" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
-        <v>249</v>
+        <v>222</v>
       </c>
     </row>
     <row r="77" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
-        <v>250</v>
+        <v>223</v>
       </c>
     </row>
     <row r="78" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
-        <v>251</v>
+        <v>224</v>
       </c>
     </row>
     <row r="79" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
-        <v>252</v>
+        <v>225</v>
       </c>
     </row>
     <row r="80" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
-        <v>253</v>
+        <v>226</v>
       </c>
     </row>
     <row r="81" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
-        <v>254</v>
+        <v>227</v>
       </c>
     </row>
     <row r="82" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
-        <v>255</v>
+        <v>228</v>
       </c>
     </row>
     <row r="83" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
-        <v>256</v>
+        <v>229</v>
       </c>
     </row>
     <row r="84" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
-        <v>257</v>
+        <v>230</v>
       </c>
     </row>
     <row r="85" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
-        <v>258</v>
+        <v>231</v>
       </c>
     </row>
     <row r="86" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
-        <v>259</v>
+        <v>232</v>
       </c>
     </row>
     <row r="87" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
-        <v>260</v>
+        <v>233</v>
       </c>
     </row>
     <row r="88" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
-        <v>261</v>
+        <v>234</v>
       </c>
     </row>
     <row r="89" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
-        <v>262</v>
+        <v>235</v>
       </c>
     </row>
     <row r="90" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
-        <v>263</v>
+        <v>236</v>
       </c>
     </row>
     <row r="91" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
-        <v>264</v>
+        <v>237</v>
       </c>
     </row>
     <row r="92" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
-        <v>265</v>
+        <v>238</v>
       </c>
     </row>
     <row r="93" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
-        <v>266</v>
+        <v>239</v>
       </c>
     </row>
     <row r="94" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
-        <v>267</v>
+        <v>240</v>
       </c>
     </row>
     <row r="95" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
-        <v>268</v>
+        <v>241</v>
       </c>
     </row>
     <row r="96" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
-        <v>210</v>
+        <v>183</v>
       </c>
     </row>
     <row r="97" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
-        <v>209</v>
+        <v>182</v>
       </c>
     </row>
     <row r="98" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
-        <v>215</v>
+        <v>188</v>
       </c>
     </row>
     <row r="99" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
-        <v>216</v>
+        <v>189</v>
       </c>
     </row>
     <row r="100" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
-        <v>269</v>
+        <v>242</v>
       </c>
     </row>
     <row r="101" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
-        <v>270</v>
+        <v>243</v>
       </c>
     </row>
     <row r="102" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
-        <v>271</v>
+        <v>244</v>
       </c>
     </row>
     <row r="103" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
-        <v>272</v>
+        <v>245</v>
       </c>
     </row>
     <row r="104" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
-        <v>273</v>
+        <v>246</v>
       </c>
     </row>
     <row r="105" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
-        <v>274</v>
+        <v>247</v>
       </c>
     </row>
     <row r="106" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
-        <v>275</v>
+        <v>248</v>
       </c>
     </row>
     <row r="107" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
-        <v>276</v>
+        <v>249</v>
       </c>
     </row>
     <row r="108" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
-        <v>277</v>
+        <v>250</v>
       </c>
     </row>
     <row r="109" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A109" t="s">
-        <v>278</v>
+        <v>251</v>
       </c>
     </row>
     <row r="110" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
-        <v>279</v>
+        <v>252</v>
       </c>
     </row>
     <row r="111" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
-        <v>280</v>
+        <v>253</v>
       </c>
     </row>
     <row r="112" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
-        <v>281</v>
+        <v>254</v>
       </c>
     </row>
     <row r="113" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
-        <v>282</v>
+        <v>255</v>
       </c>
     </row>
     <row r="114" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A114" t="s">
-        <v>283</v>
+        <v>256</v>
       </c>
     </row>
     <row r="115" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A115" t="s">
-        <v>284</v>
+        <v>257</v>
       </c>
     </row>
     <row r="116" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A116" t="s">
-        <v>285</v>
+        <v>258</v>
       </c>
     </row>
     <row r="117" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A117" t="s">
-        <v>286</v>
+        <v>259</v>
       </c>
     </row>
     <row r="118" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A118" t="s">
-        <v>287</v>
+        <v>260</v>
       </c>
     </row>
     <row r="119" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A119" t="s">
-        <v>288</v>
+        <v>261</v>
       </c>
     </row>
     <row r="120" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A120" t="s">
-        <v>289</v>
+        <v>262</v>
       </c>
     </row>
     <row r="121" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A121" t="s">
-        <v>290</v>
+        <v>263</v>
       </c>
     </row>
     <row r="122" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A122" t="s">
-        <v>291</v>
+        <v>264</v>
       </c>
     </row>
     <row r="123" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A123" t="s">
-        <v>292</v>
+        <v>265</v>
       </c>
     </row>
     <row r="124" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.3">
@@ -5047,18 +4847,18 @@
     </row>
     <row r="125" spans="1:4" ht="23.4" x14ac:dyDescent="0.3">
       <c r="A125" s="11" t="s">
-        <v>340</v>
+        <v>313</v>
       </c>
     </row>
     <row r="126" spans="1:4" ht="15" x14ac:dyDescent="0.3">
       <c r="A126" s="12" t="s">
-        <v>341</v>
+        <v>314</v>
       </c>
       <c r="B126" s="12" t="s">
-        <v>342</v>
+        <v>315</v>
       </c>
       <c r="C126" s="12" t="s">
-        <v>295</v>
+        <v>268</v>
       </c>
     </row>
     <row r="127" spans="1:4" ht="30" x14ac:dyDescent="0.3">
@@ -5066,10 +4866,10 @@
         <v>1</v>
       </c>
       <c r="B127" s="14" t="s">
-        <v>343</v>
+        <v>316</v>
       </c>
       <c r="C127" s="14" t="s">
-        <v>344</v>
+        <v>317</v>
       </c>
     </row>
     <row r="128" spans="1:4" ht="73.2" x14ac:dyDescent="0.3">
@@ -5077,10 +4877,10 @@
         <v>2</v>
       </c>
       <c r="B128" s="14" t="s">
-        <v>345</v>
+        <v>318</v>
       </c>
       <c r="C128" s="13" t="s">
-        <v>346</v>
+        <v>319</v>
       </c>
     </row>
     <row r="129" spans="1:3" ht="29.4" x14ac:dyDescent="0.3">
@@ -5088,10 +4888,10 @@
         <v>3</v>
       </c>
       <c r="B129" s="14" t="s">
-        <v>347</v>
+        <v>320</v>
       </c>
       <c r="C129" s="13" t="s">
-        <v>348</v>
+        <v>321</v>
       </c>
     </row>
     <row r="130" spans="1:3" ht="43.8" x14ac:dyDescent="0.3">
@@ -5099,10 +4899,10 @@
         <v>4</v>
       </c>
       <c r="B130" s="14" t="s">
-        <v>349</v>
+        <v>322</v>
       </c>
       <c r="C130" s="13" t="s">
-        <v>350</v>
+        <v>323</v>
       </c>
     </row>
     <row r="131" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
@@ -5110,10 +4910,10 @@
         <v>5</v>
       </c>
       <c r="B131" s="14" t="s">
-        <v>351</v>
+        <v>324</v>
       </c>
       <c r="C131" s="13" t="s">
-        <v>352</v>
+        <v>325</v>
       </c>
     </row>
     <row r="132" spans="1:3" ht="43.8" x14ac:dyDescent="0.3">
@@ -5121,10 +4921,10 @@
         <v>6</v>
       </c>
       <c r="B132" s="14" t="s">
-        <v>353</v>
+        <v>326</v>
       </c>
       <c r="C132" s="13" t="s">
-        <v>354</v>
+        <v>327</v>
       </c>
     </row>
     <row r="133" spans="1:3" ht="58.8" x14ac:dyDescent="0.3">
@@ -5132,10 +4932,10 @@
         <v>7</v>
       </c>
       <c r="B133" s="14" t="s">
-        <v>355</v>
+        <v>328</v>
       </c>
       <c r="C133" s="13" t="s">
-        <v>356</v>
+        <v>329</v>
       </c>
     </row>
     <row r="134" spans="1:3" ht="15" x14ac:dyDescent="0.3">
@@ -5143,10 +4943,10 @@
         <v>8</v>
       </c>
       <c r="B134" s="14" t="s">
-        <v>357</v>
+        <v>330</v>
       </c>
       <c r="C134" s="13" t="s">
-        <v>358</v>
+        <v>331</v>
       </c>
     </row>
     <row r="135" spans="1:3" ht="29.4" x14ac:dyDescent="0.3">
@@ -5154,10 +4954,10 @@
         <v>9</v>
       </c>
       <c r="B135" s="14" t="s">
-        <v>359</v>
+        <v>332</v>
       </c>
       <c r="C135" s="13" t="s">
-        <v>360</v>
+        <v>333</v>
       </c>
     </row>
     <row r="136" spans="1:3" ht="15" x14ac:dyDescent="0.3">
@@ -5165,10 +4965,10 @@
         <v>10</v>
       </c>
       <c r="B136" s="14" t="s">
-        <v>361</v>
+        <v>334</v>
       </c>
       <c r="C136" s="13" t="s">
-        <v>362</v>
+        <v>335</v>
       </c>
     </row>
     <row r="137" spans="1:3" ht="29.4" x14ac:dyDescent="0.3">
@@ -5176,10 +4976,10 @@
         <v>11</v>
       </c>
       <c r="B137" s="14" t="s">
-        <v>363</v>
+        <v>336</v>
       </c>
       <c r="C137" s="13" t="s">
-        <v>364</v>
+        <v>337</v>
       </c>
     </row>
     <row r="138" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
@@ -5187,10 +4987,10 @@
         <v>12</v>
       </c>
       <c r="B138" s="14" t="s">
-        <v>365</v>
+        <v>338</v>
       </c>
       <c r="C138" s="13" t="s">
-        <v>366</v>
+        <v>339</v>
       </c>
     </row>
     <row r="139" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
@@ -5198,10 +4998,10 @@
         <v>13</v>
       </c>
       <c r="B139" s="14" t="s">
-        <v>367</v>
+        <v>340</v>
       </c>
       <c r="C139" s="13" t="s">
-        <v>368</v>
+        <v>341</v>
       </c>
     </row>
     <row r="140" spans="1:3" ht="15" x14ac:dyDescent="0.3">
@@ -5209,26 +5009,26 @@
         <v>14</v>
       </c>
       <c r="B140" s="14" t="s">
-        <v>369</v>
+        <v>342</v>
       </c>
       <c r="C140" s="13" t="s">
-        <v>370</v>
+        <v>343</v>
       </c>
     </row>
     <row r="142" spans="1:3" ht="23.4" x14ac:dyDescent="0.3">
       <c r="A142" s="11" t="s">
-        <v>371</v>
+        <v>344</v>
       </c>
     </row>
     <row r="144" spans="1:3" ht="15" x14ac:dyDescent="0.3">
       <c r="A144" s="12" t="s">
-        <v>341</v>
+        <v>314</v>
       </c>
       <c r="B144" s="12" t="s">
-        <v>342</v>
+        <v>315</v>
       </c>
       <c r="C144" s="12" t="s">
-        <v>295</v>
+        <v>268</v>
       </c>
     </row>
     <row r="145" spans="1:3" ht="15" x14ac:dyDescent="0.3">
@@ -5236,10 +5036,10 @@
         <v>15</v>
       </c>
       <c r="B145" s="14" t="s">
-        <v>372</v>
+        <v>345</v>
       </c>
       <c r="C145" s="14" t="s">
-        <v>373</v>
+        <v>346</v>
       </c>
     </row>
     <row r="146" spans="1:3" ht="15" x14ac:dyDescent="0.3">
@@ -5247,10 +5047,10 @@
         <v>16</v>
       </c>
       <c r="B146" s="14" t="s">
-        <v>374</v>
+        <v>347</v>
       </c>
       <c r="C146" s="14" t="s">
-        <v>375</v>
+        <v>348</v>
       </c>
     </row>
     <row r="147" spans="1:3" ht="44.4" x14ac:dyDescent="0.3">
@@ -5258,10 +5058,10 @@
         <v>17</v>
       </c>
       <c r="B147" s="14" t="s">
-        <v>376</v>
+        <v>349</v>
       </c>
       <c r="C147" s="13" t="s">
-        <v>377</v>
+        <v>350</v>
       </c>
     </row>
     <row r="148" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
@@ -5269,26 +5069,26 @@
         <v>18</v>
       </c>
       <c r="B148" s="14" t="s">
-        <v>378</v>
+        <v>351</v>
       </c>
       <c r="C148" s="13" t="s">
-        <v>379</v>
+        <v>352</v>
       </c>
     </row>
     <row r="150" spans="1:3" ht="23.4" x14ac:dyDescent="0.3">
       <c r="A150" s="11" t="s">
-        <v>380</v>
+        <v>353</v>
       </c>
     </row>
     <row r="152" spans="1:3" ht="15" x14ac:dyDescent="0.3">
       <c r="A152" s="12" t="s">
-        <v>341</v>
+        <v>314</v>
       </c>
       <c r="B152" s="12" t="s">
-        <v>342</v>
+        <v>315</v>
       </c>
       <c r="C152" s="12" t="s">
-        <v>295</v>
+        <v>268</v>
       </c>
     </row>
     <row r="153" spans="1:3" ht="29.4" x14ac:dyDescent="0.3">
@@ -5296,10 +5096,10 @@
         <v>19</v>
       </c>
       <c r="B153" s="14" t="s">
-        <v>381</v>
+        <v>354</v>
       </c>
       <c r="C153" s="14" t="s">
-        <v>382</v>
+        <v>355</v>
       </c>
     </row>
     <row r="154" spans="1:3" ht="29.4" x14ac:dyDescent="0.3">
@@ -5307,10 +5107,10 @@
         <v>20</v>
       </c>
       <c r="B154" s="14" t="s">
-        <v>383</v>
+        <v>356</v>
       </c>
       <c r="C154" s="14" t="s">
-        <v>384</v>
+        <v>357</v>
       </c>
     </row>
     <row r="155" spans="1:3" ht="58.2" x14ac:dyDescent="0.3">
@@ -5318,26 +5118,26 @@
         <v>21</v>
       </c>
       <c r="B155" s="14" t="s">
-        <v>385</v>
+        <v>358</v>
       </c>
       <c r="C155" s="13" t="s">
-        <v>386</v>
+        <v>359</v>
       </c>
     </row>
     <row r="157" spans="1:3" ht="23.4" x14ac:dyDescent="0.3">
       <c r="A157" s="11" t="s">
-        <v>387</v>
+        <v>360</v>
       </c>
     </row>
     <row r="159" spans="1:3" ht="15" x14ac:dyDescent="0.3">
       <c r="A159" s="12" t="s">
-        <v>341</v>
+        <v>314</v>
       </c>
       <c r="B159" s="12" t="s">
-        <v>342</v>
+        <v>315</v>
       </c>
       <c r="C159" s="12" t="s">
-        <v>295</v>
+        <v>268</v>
       </c>
     </row>
     <row r="160" spans="1:3" ht="43.8" x14ac:dyDescent="0.3">
@@ -5345,10 +5145,10 @@
         <v>22</v>
       </c>
       <c r="B160" s="14" t="s">
-        <v>388</v>
+        <v>361</v>
       </c>
       <c r="C160" s="14" t="s">
-        <v>389</v>
+        <v>362</v>
       </c>
     </row>
     <row r="161" spans="1:3" ht="29.4" x14ac:dyDescent="0.3">
@@ -5356,26 +5156,26 @@
         <v>23</v>
       </c>
       <c r="B161" s="14" t="s">
-        <v>390</v>
+        <v>363</v>
       </c>
       <c r="C161" s="14" t="s">
-        <v>391</v>
+        <v>364</v>
       </c>
     </row>
     <row r="163" spans="1:3" ht="23.4" x14ac:dyDescent="0.3">
       <c r="A163" s="11" t="s">
-        <v>392</v>
+        <v>365</v>
       </c>
     </row>
     <row r="165" spans="1:3" ht="15" x14ac:dyDescent="0.3">
       <c r="A165" s="12" t="s">
-        <v>341</v>
+        <v>314</v>
       </c>
       <c r="B165" s="12" t="s">
-        <v>342</v>
+        <v>315</v>
       </c>
       <c r="C165" s="12" t="s">
-        <v>295</v>
+        <v>268</v>
       </c>
     </row>
     <row r="166" spans="1:3" ht="43.8" x14ac:dyDescent="0.3">
@@ -5383,10 +5183,10 @@
         <v>24</v>
       </c>
       <c r="B166" s="14" t="s">
-        <v>393</v>
+        <v>366</v>
       </c>
       <c r="C166" s="14" t="s">
-        <v>394</v>
+        <v>367</v>
       </c>
     </row>
     <row r="167" spans="1:3" ht="43.8" x14ac:dyDescent="0.3">
@@ -5394,26 +5194,26 @@
         <v>25</v>
       </c>
       <c r="B167" s="14" t="s">
-        <v>395</v>
+        <v>368</v>
       </c>
       <c r="C167" s="13" t="s">
-        <v>396</v>
+        <v>369</v>
       </c>
     </row>
     <row r="169" spans="1:3" ht="23.4" x14ac:dyDescent="0.3">
       <c r="A169" s="11" t="s">
-        <v>397</v>
+        <v>370</v>
       </c>
     </row>
     <row r="171" spans="1:3" ht="15" x14ac:dyDescent="0.3">
       <c r="A171" s="12" t="s">
-        <v>341</v>
+        <v>314</v>
       </c>
       <c r="B171" s="12" t="s">
-        <v>342</v>
+        <v>315</v>
       </c>
       <c r="C171" s="12" t="s">
-        <v>295</v>
+        <v>268</v>
       </c>
     </row>
     <row r="172" spans="1:3" ht="87.6" x14ac:dyDescent="0.3">
@@ -5421,10 +5221,10 @@
         <v>26</v>
       </c>
       <c r="B172" s="14" t="s">
-        <v>398</v>
+        <v>371</v>
       </c>
       <c r="C172" s="13" t="s">
-        <v>399</v>
+        <v>372</v>
       </c>
     </row>
     <row r="173" spans="1:3" ht="29.4" x14ac:dyDescent="0.3">
@@ -5432,26 +5232,26 @@
         <v>27</v>
       </c>
       <c r="B173" s="14" t="s">
-        <v>400</v>
+        <v>373</v>
       </c>
       <c r="C173" s="13" t="s">
-        <v>401</v>
+        <v>374</v>
       </c>
     </row>
     <row r="175" spans="1:3" ht="23.4" x14ac:dyDescent="0.3">
       <c r="A175" s="11" t="s">
-        <v>402</v>
+        <v>375</v>
       </c>
     </row>
     <row r="177" spans="1:3" ht="15" x14ac:dyDescent="0.3">
       <c r="A177" s="12" t="s">
-        <v>341</v>
+        <v>314</v>
       </c>
       <c r="B177" s="12" t="s">
-        <v>342</v>
+        <v>315</v>
       </c>
       <c r="C177" s="12" t="s">
-        <v>295</v>
+        <v>268</v>
       </c>
     </row>
     <row r="178" spans="1:3" ht="87.6" x14ac:dyDescent="0.3">
@@ -5459,31 +5259,31 @@
         <v>28</v>
       </c>
       <c r="B178" s="14" t="s">
-        <v>403</v>
+        <v>376</v>
       </c>
       <c r="C178" s="13" t="s">
-        <v>404</v>
+        <v>377</v>
       </c>
     </row>
     <row r="180" spans="1:3" ht="15" x14ac:dyDescent="0.35">
       <c r="A180" t="s">
-        <v>405</v>
+        <v>378</v>
       </c>
     </row>
     <row r="181" spans="1:3" ht="23.4" x14ac:dyDescent="0.3">
       <c r="A181" s="11" t="s">
-        <v>406</v>
+        <v>379</v>
       </c>
     </row>
     <row r="183" spans="1:3" ht="15" x14ac:dyDescent="0.3">
       <c r="A183" s="12" t="s">
-        <v>341</v>
+        <v>314</v>
       </c>
       <c r="B183" s="12" t="s">
-        <v>342</v>
+        <v>315</v>
       </c>
       <c r="C183" s="12" t="s">
-        <v>295</v>
+        <v>268</v>
       </c>
     </row>
     <row r="184" spans="1:3" ht="43.8" x14ac:dyDescent="0.3">
@@ -5491,10 +5291,10 @@
         <v>29</v>
       </c>
       <c r="B184" s="14" t="s">
-        <v>407</v>
+        <v>380</v>
       </c>
       <c r="C184" s="13" t="s">
-        <v>408</v>
+        <v>381</v>
       </c>
     </row>
     <row r="185" spans="1:3" ht="15" x14ac:dyDescent="0.3">
@@ -5502,10 +5302,10 @@
         <v>30</v>
       </c>
       <c r="B185" s="14" t="s">
-        <v>409</v>
+        <v>382</v>
       </c>
       <c r="C185" s="14" t="s">
-        <v>410</v>
+        <v>383</v>
       </c>
     </row>
     <row r="186" spans="1:3" ht="30" x14ac:dyDescent="0.3">
@@ -5513,10 +5313,10 @@
         <v>31</v>
       </c>
       <c r="B186" s="14" t="s">
-        <v>411</v>
+        <v>384</v>
       </c>
       <c r="C186" s="14" t="s">
-        <v>412</v>
+        <v>385</v>
       </c>
     </row>
     <row r="187" spans="1:3" ht="15" x14ac:dyDescent="0.3">
@@ -5524,10 +5324,10 @@
         <v>32</v>
       </c>
       <c r="B187" s="14" t="s">
-        <v>413</v>
+        <v>386</v>
       </c>
       <c r="C187" s="14" t="s">
-        <v>414</v>
+        <v>387</v>
       </c>
     </row>
     <row r="188" spans="1:3" ht="29.4" x14ac:dyDescent="0.3">
@@ -5535,10 +5335,10 @@
         <v>33</v>
       </c>
       <c r="B188" s="14" t="s">
-        <v>415</v>
+        <v>388</v>
       </c>
       <c r="C188" s="13" t="s">
-        <v>416</v>
+        <v>389</v>
       </c>
     </row>
     <row r="189" spans="1:3" ht="15" x14ac:dyDescent="0.3">
@@ -5546,10 +5346,10 @@
         <v>34</v>
       </c>
       <c r="B189" s="14" t="s">
-        <v>417</v>
+        <v>390</v>
       </c>
       <c r="C189" s="14" t="s">
-        <v>418</v>
+        <v>391</v>
       </c>
     </row>
     <row r="190" spans="1:3" ht="30" x14ac:dyDescent="0.3">
@@ -5557,10 +5357,10 @@
         <v>35</v>
       </c>
       <c r="B190" s="14" t="s">
-        <v>419</v>
+        <v>392</v>
       </c>
       <c r="C190" s="14" t="s">
-        <v>420</v>
+        <v>393</v>
       </c>
     </row>
     <row r="191" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
@@ -5568,10 +5368,10 @@
         <v>36</v>
       </c>
       <c r="B191" s="14" t="s">
-        <v>421</v>
+        <v>394</v>
       </c>
       <c r="C191" s="13" t="s">
-        <v>422</v>
+        <v>395</v>
       </c>
     </row>
     <row r="192" spans="1:3" ht="29.4" x14ac:dyDescent="0.3">
@@ -5579,10 +5379,10 @@
         <v>37</v>
       </c>
       <c r="B192" s="14" t="s">
-        <v>423</v>
+        <v>396</v>
       </c>
       <c r="C192" s="13" t="s">
-        <v>424</v>
+        <v>397</v>
       </c>
     </row>
     <row r="194" spans="1:1" ht="23.4" x14ac:dyDescent="0.3">
@@ -5609,16 +5409,16 @@
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
-        <v>295</v>
+        <v>268</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>298</v>
+        <v>271</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>296</v>
+        <v>269</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>297</v>
+        <v>270</v>
       </c>
       <c r="O1" s="1"/>
     </row>

</xml_diff>

<commit_message>
added docs of Abbreviated Function Templates and Lambda Improvements in Cpp20, also added blank docs for simplicity in creating new docs, also updated the xml file
</commit_message>
<xml_diff>
--- a/docs/roadmap/Roadmap - C++ New Features.xlsx
+++ b/docs/roadmap/Roadmap - C++ New Features.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git\Cpp-Modern-Features\docs\roadmap\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2635B9DF-63C8-4C39-A3CB-328679D12CB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B4525AB-A096-4A1E-957C-4E955F76F2A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="735" uniqueCount="413">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="739" uniqueCount="413">
   <si>
     <t>Hadi Abbasi</t>
   </si>
@@ -3677,18 +3677,30 @@
       <c r="B10" s="3" t="s">
         <v>0</v>
       </c>
+      <c r="C10" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>408</v>
+      </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>410</v>
+        <v>75</v>
       </c>
       <c r="B11" s="3" t="s">
         <v>0</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>408</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>411</v>
+        <v>76</v>
       </c>
       <c r="B12" s="3" t="s">
         <v>0</v>
@@ -3696,7 +3708,7 @@
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>412</v>
+        <v>77</v>
       </c>
       <c r="B13" s="3" t="s">
         <v>0</v>
@@ -3704,7 +3716,7 @@
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="B14" s="3" t="s">
         <v>0</v>
@@ -3712,7 +3724,7 @@
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="B15" s="3" t="s">
         <v>0</v>
@@ -3720,7 +3732,7 @@
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="B16" s="3" t="s">
         <v>0</v>
@@ -3728,7 +3740,7 @@
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="B17" s="3" t="s">
         <v>0</v>
@@ -3736,7 +3748,7 @@
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>80</v>
+        <v>87</v>
       </c>
       <c r="B18" s="3" t="s">
         <v>0</v>
@@ -3744,7 +3756,7 @@
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>81</v>
+        <v>88</v>
       </c>
       <c r="B19" s="3" t="s">
         <v>0</v>
@@ -3752,7 +3764,7 @@
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="B20" s="3" t="s">
         <v>0</v>
@@ -3760,7 +3772,7 @@
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>87</v>
+        <v>94</v>
       </c>
       <c r="B21" s="3" t="s">
         <v>0</v>
@@ -3768,7 +3780,7 @@
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="B22" s="3" t="s">
         <v>0</v>
@@ -3776,7 +3788,7 @@
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>89</v>
+        <v>96</v>
       </c>
       <c r="B23" s="3" t="s">
         <v>0</v>
@@ -3784,7 +3796,7 @@
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>94</v>
+        <v>55</v>
       </c>
       <c r="B24" s="3" t="s">
         <v>0</v>
@@ -3792,7 +3804,7 @@
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B25" s="3" t="s">
         <v>0</v>
@@ -3800,7 +3812,7 @@
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B26" s="3" t="s">
         <v>0</v>
@@ -3808,7 +3820,7 @@
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>55</v>
+        <v>99</v>
       </c>
       <c r="B27" s="3" t="s">
         <v>0</v>
@@ -3816,7 +3828,7 @@
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="B28" s="3" t="s">
         <v>0</v>
@@ -3824,7 +3836,7 @@
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="B29" s="3" t="s">
         <v>0</v>
@@ -3832,7 +3844,7 @@
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="B30" s="3" t="s">
         <v>0</v>
@@ -3840,7 +3852,7 @@
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="B31" s="3" t="s">
         <v>0</v>
@@ -3848,7 +3860,7 @@
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>101</v>
+        <v>410</v>
       </c>
       <c r="B32" s="3" t="s">
         <v>0</v>
@@ -3856,7 +3868,7 @@
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>102</v>
+        <v>411</v>
       </c>
       <c r="B33" s="3" t="s">
         <v>0</v>
@@ -3864,7 +3876,7 @@
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>103</v>
+        <v>412</v>
       </c>
       <c r="B34" s="3" t="s">
         <v>0</v>

</xml_diff>

<commit_message>
added docs for lambda pack captures and template lambdas in c++20
</commit_message>
<xml_diff>
--- a/docs/roadmap/Roadmap - C++ New Features.xlsx
+++ b/docs/roadmap/Roadmap - C++ New Features.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git\Cpp-Modern-Features\docs\roadmap\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B4525AB-A096-4A1E-957C-4E955F76F2A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1605A29-9983-4D51-BB69-DB51114DC572}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="739" uniqueCount="413">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="743" uniqueCount="413">
   <si>
     <t>Hadi Abbasi</t>
   </si>
@@ -3705,6 +3705,12 @@
       <c r="B12" s="3" t="s">
         <v>0</v>
       </c>
+      <c r="C12" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D12" s="7" t="s">
+        <v>408</v>
+      </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
@@ -3712,6 +3718,12 @@
       </c>
       <c r="B13" s="3" t="s">
         <v>0</v>
+      </c>
+      <c r="C13" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D13" s="7" t="s">
+        <v>408</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
added docs of std:format , std::source_location in cpp20
</commit_message>
<xml_diff>
--- a/docs/roadmap/Roadmap - C++ New Features.xlsx
+++ b/docs/roadmap/Roadmap - C++ New Features.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git\Cpp-Modern-Features\docs\roadmap\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1605A29-9983-4D51-BB69-DB51114DC572}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC00DF9C-C9A3-4E2E-99D4-2294B7C0E2B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="743" uniqueCount="413">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="747" uniqueCount="413">
   <si>
     <t>Hadi Abbasi</t>
   </si>
@@ -3733,6 +3733,12 @@
       <c r="B14" s="3" t="s">
         <v>0</v>
       </c>
+      <c r="C14" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D14" s="7" t="s">
+        <v>408</v>
+      </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
@@ -3740,6 +3746,12 @@
       </c>
       <c r="B15" s="3" t="s">
         <v>0</v>
+      </c>
+      <c r="C15" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D15" s="7" t="s">
+        <v>408</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
added docs for std::jthread and std::counting_semaphore in cpp20
</commit_message>
<xml_diff>
--- a/docs/roadmap/Roadmap - C++ New Features.xlsx
+++ b/docs/roadmap/Roadmap - C++ New Features.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git\Cpp-Modern-Features\docs\roadmap\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC00DF9C-C9A3-4E2E-99D4-2294B7C0E2B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{385395C3-BAFD-48DA-B313-A7687FAF3BCF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="747" uniqueCount="413">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="751" uniqueCount="413">
   <si>
     <t>Hadi Abbasi</t>
   </si>
@@ -3761,16 +3761,28 @@
       <c r="B16" s="3" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C16" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D16" s="7" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>86</v>
       </c>
       <c r="B17" s="3" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C17" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D17" s="7" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>87</v>
       </c>
@@ -3778,7 +3790,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>88</v>
       </c>
@@ -3786,7 +3798,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>89</v>
       </c>
@@ -3794,7 +3806,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>94</v>
       </c>
@@ -3802,7 +3814,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>95</v>
       </c>
@@ -3810,7 +3822,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>96</v>
       </c>
@@ -3818,7 +3830,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>55</v>
       </c>
@@ -3826,7 +3838,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>97</v>
       </c>
@@ -3834,7 +3846,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>98</v>
       </c>
@@ -3842,7 +3854,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>99</v>
       </c>
@@ -3850,7 +3862,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>100</v>
       </c>
@@ -3858,7 +3870,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>101</v>
       </c>
@@ -3866,7 +3878,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>102</v>
       </c>
@@ -3874,7 +3886,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>103</v>
       </c>
@@ -3882,7 +3894,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>410</v>
       </c>

</xml_diff>

<commit_message>
added docs of std::atomic<std::shared_ptr>, std::atomic<std::weak_ptr>, std::bit_cast, std::erase
</commit_message>
<xml_diff>
--- a/docs/roadmap/Roadmap - C++ New Features.xlsx
+++ b/docs/roadmap/Roadmap - C++ New Features.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git\Cpp-Modern-Features\docs\roadmap\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{385395C3-BAFD-48DA-B313-A7687FAF3BCF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9DFD31F-3FA4-4C93-A644-D49C3464FCBF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="751" uniqueCount="413">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="759" uniqueCount="413">
   <si>
     <t>Hadi Abbasi</t>
   </si>
@@ -3789,6 +3789,12 @@
       <c r="B18" s="3" t="s">
         <v>0</v>
       </c>
+      <c r="C18" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D18" s="7" t="s">
+        <v>408</v>
+      </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
@@ -3797,6 +3803,12 @@
       <c r="B19" s="3" t="s">
         <v>0</v>
       </c>
+      <c r="C19" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D19" s="7" t="s">
+        <v>408</v>
+      </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
@@ -3805,6 +3817,12 @@
       <c r="B20" s="3" t="s">
         <v>0</v>
       </c>
+      <c r="C20" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D20" s="7" t="s">
+        <v>408</v>
+      </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
@@ -3812,6 +3830,12 @@
       </c>
       <c r="B21" s="3" t="s">
         <v>0</v>
+      </c>
+      <c r="C21" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D21" s="7" t="s">
+        <v>408</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.3">

</xml_diff>